<commit_message>
AAA: Außendienst-Excel (Prioritäten A/B/C, Notizspalten) und korrigierte interne Excel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBhay9ftM7ciQ2MUqqBU5G
</commit_message>
<xml_diff>
--- a/aaa_Aussteller_Ampel.xlsx
+++ b/aaa_Aussteller_Ampel.xlsx
@@ -116,7 +116,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -583,12 +583,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sitz Engelberg 2, 88480 Achstetten. Gruppe: ACD Holding (Achstetten); ACD Elektronik GmbH (mobile Geräte, Achstetten); ACD Antriebstechnik GmbH (Safety-/Antriebstechnik, Achstetten); ACD Systemtechnik GmbH (EMS, Neustadt/Orla); ACD Czech s.r.o. (EMS/Kabel, …  [Gebiet: Baden-Württemberg (Achstetten); Gruppe hat …]</t>
+          <t>Sitz Engelberg 2, 88480 Achstetten. Gruppe: ACD Holding (Achstetten); ACD Elektronik GmbH (mobile Geräte, Achstetten); ACD Antriebstechnik GmbH (Safety-/Antriebstechnik, Achstetten); ACD Systemtechnik GmbH (EMS, Neustadt/Orla); ACD Czech s.r.o. (EMS/Kabel …</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Mittel, Stufe S. Begründung: Konzern mit Werken in Achstetten, Neustadt/Orla und Tschechien, daher V nötig. Quellen nur S: Gruppenseite führt Achstetten als Produktionsstandort (WebFetch), Schwäbische Zeitung (Artikel 2011, aktualisiert 2019): Sparte Automation komplett in Achstetten, Fertigung als Inselfertigung (WebFetch, S); …</t>
+          <t>Mittel, Stufe S. Begründung: Konzern mit Werken in Achstetten, Neustadt/Orla und Tschechien, daher V nötig. Quellen nur S: Gruppenseite führt Achstetten als Produktionsstandort (WebFetch), Schwäbische Zeitung (Artikel 2011, aktualisiert 2019): Sparte Automation komplett in Achstetten, Fertigung als Inselfertigung (WebFetch, S) …</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Steinbrüchenstraße 14, 99428 Grammetal OT Nohra (Firmenhauptsitz; Fertigung am Hauptsitz laut Presseartikel V). Niederlassungen Chemnitz und Lüdenscheid.  [Gebiet: Rest Deutschland+Niederlande (Grammetal OT Nohra, …]</t>
+          <t>Steinbrüchenstraße 14, 99428 Grammetal OT Nohra (Firmenhauptsitz; Fertigung am Hauptsitz laut Presseartikel V). Niederlassungen Chemnitz und Lüdenscheid.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sitz Westerbachstraße 7, 61476 Kronberg (V, Impressum); zweiter Standort Technologiezentrum Carl-Zeiss-Str. 72, 72770 Reutlingen (V als Adresse). Fertigung in Reutlingen laut Messe-Text und Stellenanzeigen (S).  [Gebiet: Baden-Württemberg (Fertigung im …]</t>
+          <t>Sitz Westerbachstraße 7, 61476 Kronberg (V, Impressum); zweiter Standort Technologiezentrum Carl-Zeiss-Str. 72, 72770 Reutlingen (V als Adresse). Fertigung in Reutlingen laut Messe-Text und Stellenanzeigen (S).</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -755,12 +755,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Freunder Weg 106, 52068 Aachen (Impressum, S). Entwicklung, Produktion und Kabelkonfektion laut Stellenanzeige am Standort Aachen (S).  [Gebiet: Rest Deutschland+Niederlande (Aachen, NRW)]</t>
+          <t>Freunder Weg 106, 52068 Aachen (Impressum, S). Entwicklung, Produktion und Kabelkonfektion laut Stellenanzeige am Standort Aachen (S).</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Hoch, Stufe A (Sitzregel: Hersteller mit eigener Kabelkonfektion und erkennbarem Standort Aachen, eigene Produkte; Hinweise auf Auslagerung nicht gezielt geprüft). Stützend V: Startseite "Entwicklung &amp; Fertigung KUNDENSPEZIFISCHE KABELKONFEKTION" und "Fertigung von PATCHKABEL IN SPRITZGUSSTECHNIK" (ohne Ortsangabe); S: …</t>
+          <t>Hoch, Stufe A (Sitzregel: Hersteller mit eigener Kabelkonfektion und erkennbarem Standort Aachen, eigene Produkte; Hinweise auf Auslagerung nicht gezielt geprüft). Stützend V: Startseite "Entwicklung &amp; Fertigung KUNDENSPEZIFISCHE KABELKONFEKTION" und "Fertigung von PATCHKABEL IN SPRITZGUSSTECHNIK" (ohne Ortsangabe); S …</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Neidenburger Straße 28, 28207 Bremen (Impressum, S). Ort der Hardware-Fertigung/-Montage nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Bremen); weitere …]</t>
+          <t>Neidenburger Straße 28, 28207 Bremen (Impressum, S). Ort der Hardware-Fertigung/-Montage nicht belegt.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>BAT Maschinenbau GmbH, Darmcher Grund 5, 58540 Meinerzhagen (Verzeichnis cylex/implisense, S). Fertigende Einheit: dieselbe (Sondermaschinenbauer, kein Konzern erkennbar).  [Gebiet: Rest Deutschland+Niederlande (Meinerzhagen, NRW)]</t>
+          <t>BAT Maschinenbau GmbH, Darmcher Grund 5, 58540 Meinerzhagen (Verzeichnis cylex/implisense, S). Fertigende Einheit: dieselbe (Sondermaschinenbauer, kein Konzern erkennbar).</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Marie-Curie-Str. 35-37, 40721 Hilden (S). Entwicklung und Bau der Geräte laut Messekatalog am Sitz, Schlüsselkomponenten und Kalibrierstandards im eigenen Haus (S).  [Gebiet: Rest Deutschland+Niederlande (Hilden, NRW)]</t>
+          <t>Marie-Curie-Str. 35-37, 40721 Hilden (S). Entwicklung und Bau der Geräte laut Messekatalog am Sitz, Schlüsselkomponenten und Kalibrierstandards im eigenen Haus (S).</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Otto-Hahn-Str. 7, 33161 Hövelhof (S, Verzeichnisse). Spritzguss-Fertigung am Sitz durch Stellenanzeige indiziert (S, siehe Feld 14).  [Gebiet: Rest Deutschland+Niederlande (Hövelhof, NRW)]</t>
+          <t>Otto-Hahn-Str. 7, 33161 Hövelhof (S, Verzeichnisse). Spritzguss-Fertigung am Sitz durch Stellenanzeige indiziert (S, siehe Feld 14).</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Am Drostenstück 31-33, 58507 Lüdenscheid (S, Verzeichnis onlinestreet.de). Sondermaschinenbau und Ofenbau am Sitz laut Fachpresse (S).  [Gebiet: Rest Deutschland+Niederlande (Lüdenscheid, NRW)]</t>
+          <t>Am Drostenstück 31-33, 58507 Lüdenscheid (S, Verzeichnis onlinestreet.de). Sondermaschinenbau und Ofenbau am Sitz laut Fachpresse (S).</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Brühlstraße 12, 89537 Giengen an der Brenz (S, elektroniknet-Anbieterkompass). Entwicklung und Montage der Systeme am Sitz (S, Channelpartner 2025 und Websuche-Zusammenfassung). Fertigende Einheit = EXTRA Computer GmbH selbst.  [Gebiet: Baden-Württemberg (Giengen an der Brenz)]</t>
+          <t>Brühlstraße 12, 89537 Giengen an der Brenz (S, elektroniknet-Anbieterkompass). Entwicklung und Montage der Systeme am Sitz (S, Channelpartner 2025 und Websuche-Zusammenfassung). Fertigende Einheit = EXTRA Computer GmbH selbst.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Weidachstraße 41-43, 74189 Weinsberg (S, Messe-/Verzeichnisprofile). Fertigung/Montage am Sitz (S: Arbeitsagentur-Stellenanzeigen "Monteur" und "Maschinenrichter" Weinsberg, Entwicklung am Sitz). Töchter USA/Indien/China (S). Fertigende Einheit: FIBRO …  [Gebiet: Baden-Württemberg (Weinsberg)]</t>
+          <t>Weidachstraße 41-43, 74189 Weinsberg (S, Messe-/Verzeichnisprofile). Fertigung/Montage am Sitz (S: Arbeitsagentur-Stellenanzeigen "Monteur" und "Maschinenrichter" Weinsberg, Entwicklung am Sitz). Töchter USA/Indien/China (S). Fertigende Einheit: FIBRO …</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Kapellenweg 4, 88525 Dürmentingen (S, Händlerseiten: Adresse "Kapellenweg 4, Dürmentingen"); Neubau am Sitz "größtes Bauprojekt der Firmengeschichte" (S, computer-automation.de); Triage nennt ca. 250 Mitarbeiter und Schwesterwerk Leipzig (Schlegel …  [Gebiet: Baden-Württemberg (Dürmentingen); Schwesterwerk …]</t>
+          <t>Kapellenweg 4, 88525 Dürmentingen (S, Händlerseiten: Adresse "Kapellenweg 4, Dürmentingen"); Neubau am Sitz "größtes Bauprojekt der Firmengeschichte" (S, computer-automation.de); Triage nennt ca. 250 Mitarbeiter und Schwesterwerk Leipzig (Schlegel …</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Daimlerstraße 8, 92533 Wernberg-Köblitz (S, Verzeichnisse und TÜV-SÜD-ISO-9001-Zertifikat 2025 mit gleicher Adresse). Entwicklung und Produktion am Sitz (S, bayern-international.de). Fertigende Einheit: GMK electronic design GmbH.  [Gebiet: Bayern (Wernberg-Köblitz, Oberpfalz)]</t>
+          <t>Daimlerstraße 8, 92533 Wernberg-Köblitz (S, Verzeichnisse und TÜV-SÜD-ISO-9001-Zertifikat 2025 mit gleicher Adresse). Entwicklung und Produktion am Sitz (S, bayern-international.de). Fertigende Einheit: GMK electronic design GmbH.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Alter Hellweg 70, 44379 Dortmund (S, Verzeichnis Automate/IMTS-Pavillon). Fertigende Einheit: GRIP GmbH Handhabungstechnik selbst (eigener Hersteller laut Verzeichnisprofil, S). Kein Konzern erkennbar; US-Büro Aberdeen (MD) seit 2023 (Vertrieb).  [Gebiet: Rest Deutschland+Niederlande (Dortmund, NRW)]</t>
+          <t>Alter Hellweg 70, 44379 Dortmund (S, Verzeichnis Automate/IMTS-Pavillon). Fertigende Einheit: GRIP GmbH Handhabungstechnik selbst (eigener Hersteller laut Verzeichnisprofil, S). Kein Konzern erkennbar; US-Büro Aberdeen (MD) seit 2023 (Vertrieb).</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Mittel, Stufe A. Einzelbewertung: elektrische Greifer (Motor + Controller) Mittel (A, Einschätzung aus Produkttyp), Sensorik/Näherungsschalter Mittel (A; Hoch, falls zugekauft vergossen), Kontaktmodule Mittel (A), Pneumatik-Dichtungen/Durchführungen Mittel (A), Werkzeugwechsler-Mechanik Niedrig (A). Kein Eigenverguss belegt, …</t>
+          <t>Mittel, Stufe A. Einzelbewertung: elektrische Greifer (Motor + Controller) Mittel (A, Einschätzung aus Produkttyp), Sensorik/Näherungsschalter Mittel (A; Hoch, falls zugekauft vergossen), Kontaktmodule Mittel (A), Pneumatik-Dichtungen/Durchführungen Mittel (A), Werkzeugwechsler-Mechanik Niedrig (A). Kein Eigenverguss belegt …</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Am Gut Wolf 15, 52070 Aachen (S, mehrere Listings). Fertigende Einheit: Hermann Zander GmbH &amp; Co. KG (Schaltgerätefabrik), Komplementär Zander GmbH Aachen (S, Registerbekanntmachung über North Data).  [Gebiet: Rest Deutschland+Niederlande (Aachen, NRW)]</t>
+          <t>Am Gut Wolf 15, 52070 Aachen (S, mehrere Listings). Fertigende Einheit: Hermann Zander GmbH &amp; Co. KG (Schaltgerätefabrik), Komplementär Zander GmbH Aachen (S, Registerbekanntmachung über North Data).</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Hoch, Stufe A (Produkttyp Relais/Sicherheitssensoren/RFID-Schalter nach Wissensbasis Block A). Einzelbewertung: Sicherheitsrelais Hoch (A), RFID-/Magnet-Sicherheitsschalter Hoch (A), Seilzugschalter Mittel (A), Netzteile Hoch (A, Produkt unbestätigt), Tethys IP65-Gehäuse (Strahlwasser/Staubschutz) Mittel (A, Dichtung/FIPFG), …</t>
+          <t>Hoch, Stufe A (Produkttyp Relais/Sicherheitssensoren/RFID-Schalter nach Wissensbasis Block A). Einzelbewertung: Sicherheitsrelais Hoch (A), RFID-/Magnet-Sicherheitsschalter Hoch (A), Seilzugschalter Mittel (A), Netzteile Hoch (A, Produkt unbestätigt), Tethys IP65-Gehäuse (Strahlwasser/Staubschutz) Mittel (A, Dichtung/FIPFG) …</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1424,10 +1424,14 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>INperfektion GmbH (717) | prüfenswert</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr"/>
+          <t>INperfektion GmbH</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>717</t>
+        </is>
+      </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
           <t>GRÜN (schwach, vorläufig)</t>
@@ -1435,7 +1439,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Friedrich-List-Allee 18, 41844 Wegberg (Presseindex-Snippet, S). Fertigende Einheit: INperfektion GmbH am Sitz (Eigenangabe Elektronikfertigung/Schaltschrankbau, S).  [Gebiet: Rest Deutschland+Niederlande (Wegberg, NRW)]</t>
+          <t>Friedrich-List-Allee 18, 41844 Wegberg (Presseindex-Snippet, S). Fertigende Einheit: INperfektion GmbH am Sitz (Eigenangabe Elektronikfertigung/Schaltschrankbau, S).</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1480,10 +1484,14 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Janitza electronics GmbH (114) | interessant</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
+          <t>Janitza electronics GmbH</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
           <t>GRÜN (vorläufig)</t>
@@ -1491,7 +1499,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Vor dem Polstück 6, 35633 Lahnau (Messe-Frankfurt-Verzeichnis, S). Entwicklung und Fertigung am Standort Lahnau laut Interview (S). Neubauprojekt mit zusätzlicher Produktionsfläche (industrial-production.de, S).  [Gebiet: Rest Deutschland+Niederlande (Lahnau, Hessen)]</t>
+          <t>Vor dem Polstück 6, 35633 Lahnau (Messe-Frankfurt-Verzeichnis, S). Entwicklung und Fertigung am Standort Lahnau laut Interview (S). Neubauprojekt mit zusätzlicher Produktionsfläche (industrial-production.de, S).</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1551,7 +1559,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Mönchengladbach, weiterer Standort Aachen (S). Fertigende Einheit: measX GmbH &amp; Co. KG (kein Konzern erkennbar).  [Gebiet: Rest Deutschland+Niederlande …]</t>
+          <t>Mönchengladbach, weiterer Standort Aachen (S). Fertigende Einheit: measX GmbH &amp; Co. KG (kein Konzern erkennbar).</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1611,7 +1619,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Vohwinkeler Str. 58, 42329 Wuppertal (S, it-in-germany.de/Messeprofil); Eigenentwicklung und Fertigung "in-house" laut Eigenaussage (S).  [Gebiet: Rest Deutschland+Niederlande (Wuppertal, NRW)]</t>
+          <t>Vohwinkeler Str. 58, 42329 Wuppertal (S, it-in-germany.de/Messeprofil); Eigenentwicklung und Fertigung "in-house" laut Eigenaussage (S).</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1671,7 +1679,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Felix-Wankel-Straße 11, 52351 Düren (Stellenanzeige, S); zweiter Standort seit 2019 Distelrather Straße, Düren (Firmenprofil, S). Messeliste: PLZ 52321 (Abweichung zur PLZ der Stellenanzeige 52351, siehe Feld 17).  [Gebiet: Rest Deutschland+Niederlande (Düren, NRW)]</t>
+          <t>Felix-Wankel-Straße 11, 52351 Düren (Stellenanzeige, S); zweiter Standort seit 2019 Distelrather Straße, Düren (Firmenprofil, S). Messeliste: PLZ 52321 (Abweichung zur PLZ der Stellenanzeige 52351, siehe Feld 17).</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1731,7 +1739,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand-Buisson-Str. 14, 13127 Berlin (Verzeichnisse, Messeliste, S). Entwicklung und "90 % der Produktion" am Berliner Hauptsitz (Eigenangabe laut Suchergebnis, S); Ausweitung in Berlin laut Pressemeldung "Optris expands in Berlin" (Titel im Snippet, S).  [Gebiet: Rest Deutschland+Niederlande (Berlin)]</t>
+          <t>Ferdinand-Buisson-Str. 14, 13127 Berlin (Verzeichnisse, Messeliste, S). Entwicklung und "90 % der Produktion" am Berliner Hauptsitz (Eigenangabe laut Suchergebnis, S); Ausweitung in Berlin laut Pressemeldung "Optris expands in Berlin" (Titel im Snippet, S).</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1791,7 +1799,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>München; eingetragene Adresse Augustenstraße 10-14, 80333 München (S, Snippet); "1.600 square meters of office and production space" in München (Logistik-heute-Snippet). Büros auch San Francisco und Austin (S).  [Gebiet: Bayern (München)]</t>
+          <t>München; eingetragene Adresse Augustenstraße 10-14, 80333 München (S, Snippet); "1.600 square meters of office and production space" in München (Logistik-heute-Snippet). Büros auch San Francisco und Austin (S).</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1851,7 +1859,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Lohbachstraße 14, 58239 Schwerte (OSADL-/Verzeichnis-Snippet, S); Entwicklung, Fertigung, Programmierung und Support "unter einem Dach" am deutschen Sitz (Firmenprofil-Snippet, S).  [Gebiet: Rest Deutschland+Niederlande (Schwerte, NRW)]</t>
+          <t>Lohbachstraße 14, 58239 Schwerte (OSADL-/Verzeichnis-Snippet, S); Entwicklung, Fertigung, Programmierung und Support "unter einem Dach" am deutschen Sitz (Firmenprofil-Snippet, S).</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1911,7 +1919,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Daimlerring 6, Wiesbaden (Verzeichnis-Snippet, S); Stadt Wiesbaden: Hersteller seit 2005, aktuell 20 Mitarbeitende (S). "Made in Germany" laut Gebrauchtmaschinen-Anzeige (S, schwache Quelle); Laserquelle von IPG zugekauft (Anzeige, S).  [Gebiet: Rest Deutschland+Niederlande (Wiesbaden, Hessen)]</t>
+          <t>Daimlerring 6, Wiesbaden (Verzeichnis-Snippet, S); Stadt Wiesbaden: Hersteller seit 2005, aktuell 20 Mitarbeitende (S). "Made in Germany" laut Gebrauchtmaschinen-Anzeige (S, schwache Quelle); Laserquelle von IPG zugekauft (Anzeige, S).</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1956,10 +1964,14 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>W. Gessmann GmbH (Stand 806) | interessant</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
+          <t>W. Gessmann GmbH</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>806</t>
+        </is>
+      </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
           <t>GRÜN (vorläufig, kein V)</t>
@@ -1967,7 +1979,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Eppingerstr. 221, 74211 Leingarten (S, Katalog/Verzeichnis); laut Triage Entwicklung, Teilmontage, CNC, THT/SMD im Werk Leingarten (S, plantautomation-technology.com, nicht erneut gelesen). Tochter Gessmann China Ltd. (Shanghai) laut Triage: Fertigungsrolle …  [Gebiet: Baden-Württemberg (Leingarten)]</t>
+          <t>Eppingerstr. 221, 74211 Leingarten (S, Katalog/Verzeichnis); laut Triage Entwicklung, Teilmontage, CNC, THT/SMD im Werk Leingarten (S, plantautomation-technology.com, nicht erneut gelesen). Tochter Gessmann China Ltd. (Shanghai) laut Triage: Fertigungsrolle …</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -2027,7 +2039,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Heidelberg (Hauptstandort einschließlich Produktion, V); weitere Elektronikproduktion in Hornberg (V). Fertigende Einheit laut ABB-Seite: "ABB AG" unter der Marke STOTZ-KONTAKT (siehe Feld 17).  [Gebiet: Baden-Württemberg (Heidelberg und Hornberg)]</t>
+          <t>Heidelberg (Hauptstandort einschließlich Produktion, V); weitere Elektronikproduktion in Hornberg (V). Fertigende Einheit laut ABB-Seite: "ABB AG" unter der Marke STOTZ-KONTAKT (siehe Feld 17).</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -2087,7 +2099,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Sitz Werner-von-Siemens-Straße 16-18, 65582 Diez (V, Impressum). Werk Diez (Accuride Germany, Teil einer Gruppe mit weiteren Werken, siehe Feld 7).  [Gebiet: Rest Deutschland+Niederlande (Diez, …]</t>
+          <t>Sitz Werner-von-Siemens-Straße 16-18, 65582 Diez (V, Impressum). Werk Diez (Accuride Germany, Teil einer Gruppe mit weiteren Werken, siehe Feld 7).</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -2147,7 +2159,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Sitz laut Messeliste 80636 München; Adresse der elunic AG: Erika-Mann-Str. 23, 80636 München (S). Fertigungsort der Hardware: nicht belegt.  [Gebiet: Bayern (München; Labor Obernburg am Main …]</t>
+          <t>Sitz laut Messeliste 80636 München; Adresse der elunic AG: Erika-Mann-Str. 23, 80636 München (S). Fertigungsort der Hardware: nicht belegt.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -2207,7 +2219,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Schwarzwaldstr. 10, 78652 Deißlingen (Impressum, S). Fertigungsort: Messe-Text und Verzeichnisse sagen "entwickelt und fertigt", ohne Ortsangabe (S).  [Gebiet: Baden-Württemberg (Deißlingen)]</t>
+          <t>Schwarzwaldstr. 10, 78652 Deißlingen (Impressum, S). Fertigungsort: Messe-Text und Verzeichnisse sagen "entwickelt und fertigt", ohne Ortsangabe (S).</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2267,7 +2279,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Asyril GmbH, Max-Planck-Straße 1, Offenburg = Technikzentrum/Showroom seit Oktober 2023 (S). Fertigende Einheit laut Snippets: Asyril SA, Z.I. du Vivier 22, 1690 Villaz-St-Pierre (Schweiz). Fertigung der Asycube in Offenburg: nicht belegt.  [Gebiet: Baden-Württemberg (GmbH in Offenburg); …]</t>
+          <t>Asyril GmbH, Max-Planck-Straße 1, Offenburg = Technikzentrum/Showroom seit Oktober 2023 (S). Fertigende Einheit laut Snippets: Asyril SA, Z.I. du Vivier 22, 1690 Villaz-St-Pierre (Schweiz). Fertigung der Asycube in Offenburg: nicht belegt.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -2327,7 +2339,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Intzestraße 50, 42859 Remscheid (Verzeichnisse, S). Fertigungsort: nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Remscheid, NRW)]</t>
+          <t>Intzestraße 50, 42859 Remscheid (Verzeichnisse, S). Fertigungsort: nicht belegt.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2387,7 +2399,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Amberg, An den Franzosenäckern 11, 92224 Amberg (ProvenExpert, Bayern International, S). Fertigende Einheit: AUTEC Sondermaschinenbau GmbH (Teil der inhabergeführten AUTEC Gruppe, Hauptsitz Amberg, S).  [Gebiet: Bayern (Amberg)]</t>
+          <t>Amberg, An den Franzosenäckern 11, 92224 Amberg (ProvenExpert, Bayern International, S). Fertigende Einheit: AUTEC Sondermaschinenbau GmbH (Teil der inhabergeführten AUTEC Gruppe, Hauptsitz Amberg, S).</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -2402,7 +2414,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation / E-Mobility Potting (Endprodukt: Montage-/Prüfautomaten mit verbauten Antrieben, Sensorik, Steuerungen); …</t>
+          <t>Electrical Insulation / E-Mobility Potting (Endprodukt: Montage-/Prüfautomaten mit verbauten Antrieben, Sensorik, Steuerungen) …</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2447,7 +2459,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Max-Planck-Straße 34, 71116 Gärtringen (Verzeichnis, S). Fertigungsort: nicht belegt.  [Gebiet: Baden-Württemberg (Gärtringen)]</t>
+          <t>Max-Planck-Straße 34, 71116 Gärtringen (Verzeichnis, S). Fertigungsort: nicht belegt.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2507,12 +2519,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>BENEDICT GmbH, Lieblgasse 7, 1220 Wien (Wirtschaftskammer-/Advantage-Austria- und Firmenbuch-Snippet, S). Ein Profil nennt "headquarters and production lines located in Vienna" (S). Wülfrath: kein Beleg.  [Gebiet: Österreich (Wien); Messeliste nennt Wülfrath, …]</t>
+          <t>BENEDICT GmbH, Lieblgasse 7, 1220 Wien (Wirtschaftskammer-/Advantage-Austria- und Firmenbuch-Snippet, S). Ein Profil nennt "headquarters and production lines located in Vienna" (S). Wülfrath: kein Beleg.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Hoch, Stufe A (Sitzregel: eigener Gerätebauer mit erkennbarem Standort, Familien-GmbH 100 Prozent im Familienbesitz (S), eigene Produkte, kein Händler; kein Hinweis auf Auslagerung). Ergänzend S: "headquarters and production lines located in Vienna". Hinweis: Ein Konzern- oder Mehrwerkscharakter ist nicht belegt; falls doch, …</t>
+          <t>Hoch, Stufe A (Sitzregel: eigener Gerätebauer mit erkennbarem Standort, Familien-GmbH 100 Prozent im Familienbesitz (S), eigene Produkte, kein Händler; kein Hinweis auf Auslagerung). Ergänzend S: "headquarters and production lines located in Vienna". Hinweis: Ein Konzern- oder Mehrwerkscharakter ist nicht belegt; falls doch …</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2567,7 +2579,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Arbachtalstraße 26, 72800 Eningen (Verzeichnisse, S); ältere Adresse Harretstraße 1 (Berghof Automationstechnik GmbH). Katalog 2024 laut Suchzusammenfassung: Entwicklung, Produktion und Test am Hauptsitz Eningen gebündelt (S). Fertigende Einheit: Berghof …  [Gebiet: Baden-Württemberg (Eningen unter Achalm)]</t>
+          <t>Arbachtalstraße 26, 72800 Eningen (Verzeichnisse, S); ältere Adresse Harretstraße 1 (Berghof Automationstechnik GmbH). Katalog 2024 laut Suchzusammenfassung: Entwicklung, Produktion und Test am Hauptsitz Eningen gebündelt (S). Fertigende Einheit: Berghof …</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2627,12 +2639,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Maarweg 33, 53619 Rheinbreitbach (Pressemitteilung, S). Laut Bionity-Profil "develop, design and produce" am Sitz (S); Gruppe BluhmWeber mit weiteren Produktions-/Vertriebsstandorten in Europa (GS1-Profil, S).  [Gebiet: Rest Deutschland+Niederlande (Rheinbreitbach, …]</t>
+          <t>Maarweg 33, 53619 Rheinbreitbach (Pressemitteilung, S). Laut Bionity-Profil "develop, design and produce" am Sitz (S); Gruppe BluhmWeber mit weiteren Produktions-/Vertriebsstandorten in Europa (GS1-Profil, S).</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Mittel, Stufe S. Begründung: Sitz und Entwicklung/Produktion laut Profil in Rheinbreitbach, jedoch BluhmWeber-Gruppe mit mehreren Standorten (Konzernfall, V nötig); Stellenanzeigen Rheinbreitbach (Entwicklung Inkjet, Produktionsplanung/Auftragssteuerung, S) deuten auf Eigenfertigung, belegen aber Fertigungstiefe nicht. …</t>
+          <t>Mittel, Stufe S. Begründung: Sitz und Entwicklung/Produktion laut Profil in Rheinbreitbach, jedoch BluhmWeber-Gruppe mit mehreren Standorten (Konzernfall, V nötig); Stellenanzeigen Rheinbreitbach (Entwicklung Inkjet, Produktionsplanung/Auftragssteuerung, S) deuten auf Eigenfertigung, belegen aber Fertigungstiefe nicht …</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2687,7 +2699,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Wuppertal laut Messeliste (42329 Wuppertal), keine Quelle gefunden. Fertigungsort: unbekannt.  [Gebiet: Rest Deutschland+Niederlande (Wuppertal laut …]</t>
+          <t>Wuppertal laut Messeliste (42329 Wuppertal), keine Quelle gefunden. Fertigungsort: unbekannt.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2747,7 +2759,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Porschestraße 1, 73095 Albershausen (Verzeichnisse, S). Fertigung am Standort Albershausen: nicht belegt. Gruppe Camozzi (Brescia, IT) mit mehreren Produktionswerken (17 bis 25 laut unterschiedlichen Quellen, S).  [Gebiet: Baden-Württemberg (Albershausen); Konzern …]</t>
+          <t>Porschestraße 1, 73095 Albershausen (Verzeichnisse, S). Fertigung am Standort Albershausen: nicht belegt. Gruppe Camozzi (Brescia, IT) mit mehreren Produktionswerken (17 bis 25 laut unterschiedlichen Quellen, S).</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2807,7 +2819,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Industriestr. 6, 64653 Lorsch (S, Verzeichnis dasoertliche.de laut Suchtool). Die Stellenanzeige nennt "DFS Maschinenbau GmbH" (Namensvariante, Feld 17).  [Gebiet: Rest Deutschland+Niederlande (Lorsch, Hessen)]</t>
+          <t>Industriestr. 6, 64653 Lorsch (S, Verzeichnis dasoertliche.de laut Suchtool). Die Stellenanzeige nennt "DFS Maschinenbau GmbH" (Namensvariante, Feld 17).</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2867,7 +2879,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Vohwinkelallee 8, 40229 Düsseldorf (S, Pressemitteilung und Analog-Devices-Partnerseite). Ob die Module im Haus gefertigt oder extern bestückt werden, ist NICHT belegt.  [Gebiet: Rest Deutschland+Niederlande (Düsseldorf, NRW)]</t>
+          <t>Vohwinkelallee 8, 40229 Düsseldorf (S, Pressemitteilung und Analog-Devices-Partnerseite). Ob die Module im Haus gefertigt oder extern bestückt werden, ist NICHT belegt.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -2927,7 +2939,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Göppingen und Essen (S, Messeprofil); Schaltschrank-/Schaltanlagenbau laut Profil, Standortzuordnung der Fertigung nicht belegt. Einheit: Dussmann Elektrotechnik und Automation GmbH, Teil der Dussmann Technical Solutions Division seit 2025 (S).  [Gebiet: Baden-Württemberg (Göppingen); zweiter Standort …]</t>
+          <t>Göppingen und Essen (S, Messeprofil); Schaltschrank-/Schaltanlagenbau laut Profil, Standortzuordnung der Fertigung nicht belegt. Einheit: Dussmann Elektrotechnik und Automation GmbH, Teil der Dussmann Technical Solutions Division seit 2025 (S).</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2987,7 +2999,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>EFCO Electronics GmbH, Deggendorf (S, Messeprofil/Fachpresse): Design-in-Support vor Ort und Auslieferung kundenspezifischer Computer in kleinen Stückzahlen; Lieferung "aus der Zentrale in Taiwan" möglich. Fertigung der Geräte in Deutschland NICHT belegt, …  [Gebiet: Bayern (Deggendorf); Konzern EFCO Technology mit …]</t>
+          <t>EFCO Electronics GmbH, Deggendorf (S, Messeprofil/Fachpresse): Design-in-Support vor Ort und Auslieferung kundenspezifischer Computer in kleinen Stückzahlen; Lieferung "aus der Zentrale in Taiwan" möglich. Fertigung der Geräte in Deutschland NICHT belegt …</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -3047,7 +3059,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Am Johannisberg 59a, 53474 Bad Neuenahr-Ahrweiler (S, automa.net); ein zweiter Datensatz nennt Keltenweg 2e, 55288 Armsheim, HRB 52664 Mainz (S, Implisense). Fertigungsort unbekannt.  [Gebiet: Rest Deutschland+Niederlande (Rheinland-Pfalz; …]</t>
+          <t>Am Johannisberg 59a, 53474 Bad Neuenahr-Ahrweiler (S, automa.net); ein zweiter Datensatz nennt Keltenweg 2e, 55288 Armsheim, HRB 52664 Mainz (S, Implisense). Fertigungsort unbekannt.</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3107,7 +3119,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Elberfelder Straße 32, 58553 Halver (S, mehrere Verzeichnisse). Produktionsstandorte auf drei Kontinenten laut Karriereseite (S), also Gruppe mit mehreren Werken; Fertigung gerade in Halver nicht einzeln belegt.  [Gebiet: Rest Deutschland+Niederlande (Halver, NRW)]</t>
+          <t>Elberfelder Straße 32, 58553 Halver (S, mehrere Verzeichnisse). Produktionsstandorte auf drei Kontinenten laut Karriereseite (S), also Gruppe mit mehreren Werken; Fertigung gerade in Halver nicht einzeln belegt.</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -3167,7 +3179,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Hanau (S, Messeprofil MAWI Technik, Stellenanzeigen). Kalibrierlabor DAkkS-akkreditiert (D-K-15055-01-00 laut Messeprofil, S). Eigene Gerätefertigung nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Hanau, Hessen)]</t>
+          <t>Hanau (S, Messeprofil MAWI Technik, Stellenanzeigen). Kalibrierlabor DAkkS-akkreditiert (D-K-15055-01-00 laut Messeprofil, S). Eigene Gerätefertigung nicht belegt.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3227,7 +3239,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Sitz Rehwinkel 30, 32457 Porta Westfalica (S, Verzeichnisse). Fertigung DE nicht belegt. Gruppe: Fibox Oy Ab, Espoo (Finnland), Spritzguss PAM in Lempäälä (FI), Montage Kiuruvesi (FI), Fibox Sp. z o.o. Warschau (PL, Schaltschrankmontage/Kabelbäume), Fibox …  [Gebiet: Rest Deutschland+Niederlande (Sitz Porta …]</t>
+          <t>Sitz Rehwinkel 30, 32457 Porta Westfalica (S, Verzeichnisse). Fertigung DE nicht belegt. Gruppe: Fibox Oy Ab, Espoo (Finnland), Spritzguss PAM in Lempäälä (FI), Montage Kiuruvesi (FI), Fibox Sp. z o.o. Warschau (PL, Schaltschrankmontage/Kabelbäume), Fibox …</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -3287,7 +3299,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Sitz Neckarsulm (S, Verzeichnisse). Gruppe mit sieben Produktionsstätten, neun Vertriebsniederlassungen (S, Zusammenfassung der Unternehmensdarstellung). Fertigung Neckarsulm: Stellenanzeige "Produktionsleitung" für kabelgebundene und konfektionierbare …  [Gebiet: Baden-Württemberg (Neckarsulm)]</t>
+          <t>Sitz Neckarsulm (S, Verzeichnisse). Gruppe mit sieben Produktionsstätten, neun Vertriebsniederlassungen (S, Zusammenfassung der Unternehmensdarstellung). Fertigung Neckarsulm: Stellenanzeige "Produktionsleitung" für kabelgebundene und konfektionierbare …</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3347,7 +3359,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Stahlschmidtsbrücke 61, 42499 Hückeswagen laut Produktdatenblättern der Firma; Verzeichnis nennt Nr. 38 (Abweichung, S). "Vertrieb und Produktion" laut Verzeichnis it-in-germany.de (S). Eigenfertigungsumfang NICHT belegt.  [Gebiet: Rest Deutschland+Niederlande (Hückeswagen, NRW)]</t>
+          <t>Stahlschmidtsbrücke 61, 42499 Hückeswagen laut Produktdatenblättern der Firma; Verzeichnis nennt Nr. 38 (Abweichung, S). "Vertrieb und Produktion" laut Verzeichnis it-in-germany.de (S). Eigenfertigungsumfang NICHT belegt.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -3407,7 +3419,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Dresden (S: computer-automation.de, startupvalley.news; Angabe "Start-up aus Dresden, 2023 als Ausgründung aus der TU Dresden gegründet", Geschäftsführer Dr. Lucas Scheuvens). Fertigungsort der Hardware NICHT belegt.  [Gebiet: Rest Deutschland+Niederlande (Dresden, Sachsen)]</t>
+          <t>Dresden (S: computer-automation.de, startupvalley.news; Angabe "Start-up aus Dresden, 2023 als Ausgründung aus der TU Dresden gegründet", Geschäftsführer Dr. Lucas Scheuvens). Fertigungsort der Hardware NICHT belegt.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3467,7 +3479,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Lehmkuhlenweg 16, 41065 Mönchengladbach (S, Verzeichnisse). Fertigungsort der Geräte NICHT belegt (Verzeichnis: "Entwickler von Industrie-Computern und Messtechnik").  [Gebiet: Rest Deutschland+Niederlande (Mönchengladbach, …]</t>
+          <t>Lehmkuhlenweg 16, 41065 Mönchengladbach (S, Verzeichnisse). Fertigungsort der Geräte NICHT belegt (Verzeichnis: "Entwickler von Industrie-Computern und Messtechnik").</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3527,7 +3539,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Theodor-Heuss-Str. 35, 61118 Bad Vilbel (S, Verzeichnis; seit 1993 in Bad Vilbel). Eigenfertigung unklar: "Sonderversionen im Rahmen der Fertigungsmöglichkeiten", Zubehörsparte für Schaltschrankbau, Tragschienen-Zuschnitt/-Stanzung (S, …  [Gebiet: Rest Deutschland+Niederlande (Bad Vilbel, Hessen)]</t>
+          <t>Theodor-Heuss-Str. 35, 61118 Bad Vilbel (S, Verzeichnis; seit 1993 in Bad Vilbel). Eigenfertigung unklar: "Sonderversionen im Rahmen der Fertigungsmöglichkeiten", Zubehörsparte für Schaltschrankbau, Tragschienen-Zuschnitt/-Stanzung (S …</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3587,7 +3599,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Am Stadtwalde 12, 48432 Rheine (S, jobvoting.de). Schaltanlagen- und Steuerungsbau am Sitz (S, Firmenflyer/Profil). Fertigende Einheit: Hardy Schmitz GmbH &amp; Co. KG (Sparte Schaltanlagenbau); Konzern mit sechs Standorten, Holding Hardy Schmitz Holding GmbH.  [Gebiet: Rest Deutschland+Niederlande (Rheine, NRW)]</t>
+          <t>Am Stadtwalde 12, 48432 Rheine (S, jobvoting.de). Schaltanlagen- und Steuerungsbau am Sitz (S, Firmenflyer/Profil). Fertigende Einheit: Hardy Schmitz GmbH &amp; Co. KG (Sparte Schaltanlagenbau); Konzern mit sechs Standorten, Holding Hardy Schmitz Holding GmbH.</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -3597,7 +3609,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Niedrig, Stufe A. Einzelbewertung: Schaltanlagenmontage (Verdrahten, Zusammenbau) Niedrig (A), eingebaute Netzteile Mittel (A, Zukauf, nicht von der Firma vergossen), Schaltschrank-Türdichtungen Mittel (A, typischerweise Zukaufteil, FIPFG nur bei eigener Gehäusefertigung), ModCenter-Gehäusebearbeitung Niedrig (A; …</t>
+          <t>Niedrig, Stufe A. Einzelbewertung: Schaltanlagenmontage (Verdrahten, Zusammenbau) Niedrig (A), eingebaute Netzteile Mittel (A, Zukauf, nicht von der Firma vergossen), Schaltschrank-Türdichtungen Mittel (A, typischerweise Zukaufteil, FIPFG nur bei eigener Gehäusefertigung), ModCenter-Gehäusebearbeitung Niedrig (A …</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3647,7 +3659,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Kohlfurther Brücke 69, 42349 Wuppertal-Cronenberg (S, Verzeichnisse). Handelsregister Amtsgericht Wuppertal HRA 13527 (S, North Data/Verzeichnis); Komplementärin Berger Gruppe GmbH, HRB 3880 (S, Impressum-Block auf IndustryArena für eine Schwesterfirma). …  [Gebiet: Rest Deutschland+Niederlande (Wuppertal, NRW)]</t>
+          <t>Kohlfurther Brücke 69, 42349 Wuppertal-Cronenberg (S, Verzeichnisse). Handelsregister Amtsgericht Wuppertal HRA 13527 (S, North Data/Verzeichnis); Komplementärin Berger Gruppe GmbH, HRB 3880 (S, Impressum-Block auf IndustryArena für eine Schwesterfirma) …</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3707,7 +3719,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Sitz/Logistik Hemmingen (Triage-Quelle); Kabelfertigung Windsbach (Bayern, seit 1988) und Meißen (Sachsen, Balzer Kabel), außerdem Polen und China (S, Werksseite Helukabel/Presse). Konfektion: Standort nicht belegt. Fertigende Einheit für Kabel: HELUKABEL …  [Gebiet: Bayern (Fertigungsort Windsbach); Sitz Hemmingen …]</t>
+          <t>Sitz/Logistik Hemmingen (Triage-Quelle); Kabelfertigung Windsbach (Bayern, seit 1988) und Meißen (Sachsen, Balzer Kabel), außerdem Polen und China (S, Werksseite Helukabel/Presse). Konfektion: Standort nicht belegt. Fertigende Einheit für Kabel: HELUKABEL …</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -3767,7 +3779,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Karlsruhe (Niederlassung der HMS Industrial Networks GmbH, nur als Vertriebs-/Gruppenstandort belegt, S); HMS Technology Center Ravensburg (frühere Ixxat) als Entwicklungs-/Produktmanagementstandort (S). Fertigung der Gruppe: Halmstad (Schweden) als …  [Gebiet: Baden-Württemberg (Karlsruhe, Ravensburg)]</t>
+          <t>Karlsruhe (Niederlassung der HMS Industrial Networks GmbH, nur als Vertriebs-/Gruppenstandort belegt, S); HMS Technology Center Ravensburg (frühere Ixxat) als Entwicklungs-/Produktmanagementstandort (S). Fertigung der Gruppe: Halmstad (Schweden) als …</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -3827,7 +3839,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>In Laisen 74, Reutlingen (S, Fraunhofer-Datenbank/Messeprofile). Fertigende Einheit: HSB Automation GmbH selbst ("Entwicklung, Produktion und Vertrieb unter einem Dach", S, Messeprofil). Kein Konzern erkennbar. Gegründet 1993.  [Gebiet: Baden-Württemberg (Reutlingen)]</t>
+          <t>In Laisen 74, Reutlingen (S, Fraunhofer-Datenbank/Messeprofile). Fertigende Einheit: HSB Automation GmbH selbst ("Entwicklung, Produktion und Vertrieb unter einem Dach", S, Messeprofil). Kein Konzern erkennbar. Gegründet 1993.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -3887,7 +3899,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Waldkirch im Schwarzwald (S, Messeprofile, HUGRO-Katalog). "Serienfertigung" laut Messeprofil (Triage, S). Fertigende Einheit nicht ausdrücklich benannt. Selbstbeschreibung als "Swiss-German company"; Konzernzugehörigkeit unbekannt.  [Gebiet: Baden-Württemberg (Waldkirch)]</t>
+          <t>Waldkirch im Schwarzwald (S, Messeprofile, HUGRO-Katalog). "Serienfertigung" laut Messeprofil (Triage, S). Fertigende Einheit nicht ausdrücklich benannt. Selbstbeschreibung als "Swiss-German company"; Konzernzugehörigkeit unbekannt.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -3947,7 +3959,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Freudenberg (Siegerland, NRW; S, Messeprofil, Implisense). Sondermaschinenbau am Sitz nur aus Selbstbeschreibung des Messeprofils (S). Fertigende Einheit nicht eindeutig (siehe Feld 17).  [Gebiet: Rest Deutschland+Niederlande (Freudenberg, NRW)]</t>
+          <t>Freudenberg (Siegerland, NRW; S, Messeprofil, Implisense). Sondermaschinenbau am Sitz nur aus Selbstbeschreibung des Messeprofils (S). Fertigende Einheit nicht eindeutig (siehe Feld 17).</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -4007,7 +4019,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Vasco-da-Gama-Straße, 53881 Euskirchen (Großbüllesheim) (S, Verzeichnis werkenntdenbesten.de). Fertigungsort: keine Fertigung belegt.  [Gebiet: Rest Deutschland+Niederlande (Euskirchen, NRW)]</t>
+          <t>Vasco-da-Gama-Straße, 53881 Euskirchen (Großbüllesheim) (S, Verzeichnis werkenntdenbesten.de). Fertigungsort: keine Fertigung belegt.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -4052,10 +4064,14 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>igus GmbH (603) | interessant</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr"/>
+          <t>igus GmbH</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>603</t>
+        </is>
+      </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -4063,7 +4079,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Köln (Stammsitz mit Spritzguss- und Leitungsfertigung, S). Fertigende Einheit: igus-Werk Köln; Rechtsform laut Quellen schwankend igus GmbH / igus SE &amp; Co. KG (siehe Feld 17). Weltweiter Konzern mit weiteren Werken.  [Gebiet: Rest Deutschland+Niederlande (Köln, NRW)]</t>
+          <t>Köln (Stammsitz mit Spritzguss- und Leitungsfertigung, S). Fertigende Einheit: igus-Werk Köln; Rechtsform laut Quellen schwankend igus GmbH / igus SE &amp; Co. KG (siehe Feld 17). Weltweiter Konzern mit weiteren Werken.</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -4088,7 +4104,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>(a) Werden Schrittmotoren (NEMA 17/23), Encoder-/Sensorelektronik und konfektionierte Leitungen/Stecker in Köln (oder Rest DE) gefertigt und wo ist die Vergussstufe? Wo nachsehen: igus.de Produktseite Schrittmotoren/Datenblatt (Herkunftsland, "Made in"), igus-Karriereseite Köln (Montage Elektronik/Konfektion 2025/2026), Pressemeldungen zur Kölner Produktion. (b) Impressum igus.de: igus GmbH oder igus SE &amp; Co. KG, Registerauszug (Amtsgericht Köln). (c) Aktuelle V-Quelle (2025/2026) für Fertigung am Kölner Werk. …</t>
+          <t>(a) Werden Schrittmotoren (NEMA 17/23), Encoder-/Sensorelektronik und konfektionierte Leitungen/Stecker in Köln (oder Rest DE) gefertigt und wo ist die Vergussstufe? Wo nachsehen: igus.de Produktseite Schrittmotoren/Datenblatt (Herkunftsland, "Made in"), igus-Karriereseite Köln (Montage Elektronik/Konfektion 2025/2026), Pressemeldungen zur Kölner Produktion. (b) Impressum igus.de: igus GmbH oder igus SE &amp; Co. KG, Registerauszug (Amtsgericht Köln). (c) Aktuelle V-Quelle (2025/2026) für Fertigung am Kölner Werk …</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
@@ -4108,10 +4124,14 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>ima-tec GmbH (140) | prüfenswert</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr"/>
+          <t>ima-tec GmbH</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -4119,7 +4139,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Wachtelberg 10 a, 97273 Kürnach (Implisense-Snippet, S); Fertigungsort = Sitz laut Eigenbeschreibung Sondermaschinenbau (S). Seit 2017 Tochter der SAR Group (Österreich).  [Gebiet: Bayern (Kürnach bei Würzburg)]</t>
+          <t>Wachtelberg 10 a, 97273 Kürnach (Implisense-Snippet, S); Fertigungsort = Sitz laut Eigenbeschreibung Sondermaschinenbau (S). Seit 2017 Tochter der SAR Group (Österreich).</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -4164,10 +4184,14 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>IMPADY (818) | kein Fertiger</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr"/>
+          <t>IMPADY</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>818</t>
+        </is>
+      </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -4175,7 +4199,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Sitz laut Startbase: Darmstadt (S, unclaimed Profil). Vorgabe-Sitz Hoppstädten-Weiersbach (Rheinland-Pfalz): keine Quelle gefunden, die IMPADY dort nennt. Fertigungsort: nicht belegt.  [Gebiet: außerhalb/unklar (Sitz Darmstadt laut Startbase = …]</t>
+          <t>Sitz laut Startbase: Darmstadt (S, unclaimed Profil). Vorgabe-Sitz Hoppstädten-Weiersbach (Rheinland-Pfalz): keine Quelle gefunden, die IMPADY dort nennt. Fertigungsort: nicht belegt.</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -4220,10 +4244,14 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>INSEVIS GmbH (615) | prüfenswert</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr"/>
+          <t>INSEVIS GmbH</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>615</t>
+        </is>
+      </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -4231,7 +4259,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Erlangen. Anschrift der Holding laut LEI-Snippet: INSEVIS Holding GmbH, Am Weichselgarten 7, 91058 Erlangen (HRB 20784 Fürth). Fertigungsort der Geräte: NICHT belegt (nur Werbeaussage "made in Germany").  [Gebiet: Bayern (Erlangen)]</t>
+          <t>Erlangen. Anschrift der Holding laut LEI-Snippet: INSEVIS Holding GmbH, Am Weichselgarten 7, 91058 Erlangen (HRB 20784 Fürth). Fertigungsort der Geräte: NICHT belegt (nur Werbeaussage "made in Germany").</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -4276,10 +4304,14 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>IXON B.V. (438) | unwahrscheinlich</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr"/>
+          <t>IXON B.V.</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>438</t>
+        </is>
+      </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -4287,7 +4319,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Zuster Bloemstraat 20, 5835 DW Beugen, Niederlande (Händlerverzeichnis-Snippet, S). Triage nennt Overloon; Overloon in keiner Suchquelle belegt. Fertigungsort der Hardware: NICHT belegt.  [Gebiet: Rest Deutschland+Niederlande (Niederlande)]</t>
+          <t>Zuster Bloemstraat 20, 5835 DW Beugen, Niederlande (Händlerverzeichnis-Snippet, S). Triage nennt Overloon; Overloon in keiner Suchquelle belegt. Fertigungsort der Hardware: NICHT belegt.</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -4332,10 +4364,14 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>JAM automation GmbH (118) | prüfenswert</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr"/>
+          <t>JAM automation GmbH</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -4343,7 +4379,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Albert-Einstein-Str. 6, 42477 Radevormwald (Messeverzeichnis-Snippet, S). Fertigung = Sitz (Sondermaschinenbau, S). Triage-Vorgabe "Köln" ist nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Radevormwald, NRW)]</t>
+          <t>Albert-Einstein-Str. 6, 42477 Radevormwald (Messeverzeichnis-Snippet, S). Fertigung = Sitz (Sondermaschinenbau, S). Triage-Vorgabe "Köln" ist nicht belegt.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -4388,10 +4424,14 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Kaiser GmbH &amp; Co. KG (115) | prüfenswert</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr"/>
+          <t>Kaiser GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -4399,7 +4439,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Ramsloh 4, 58579 Schalksmühle (Messe-Frankfurt-Snippet, S). Fertigung am Sitz: Stellenanzeige Schalksmühle sucht Einrichter für Spritzgießmaschinen (Arburg, Engel; StepStone-Snippet, S). Weitere Standorte (4 europäische laut Triage) und Töchter AGRO (CH), …  [Gebiet: Rest Deutschland+Niederlande (Schalksmühle, NRW)]</t>
+          <t>Ramsloh 4, 58579 Schalksmühle (Messe-Frankfurt-Snippet, S). Fertigung am Sitz: Stellenanzeige Schalksmühle sucht Einrichter für Spritzgießmaschinen (Arburg, Engel; StepStone-Snippet, S). Weitere Standorte (4 europäische laut Triage) und Töchter AGRO (CH) …</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -4444,10 +4484,14 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Kalitec Verbindungstechnik GmbH (143) | kein Fertiger</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr"/>
+          <t>Kalitec Verbindungstechnik GmbH</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -4455,7 +4499,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Lindgesfeld 8h, 42653 Solingen (Telefonbuch-Snippet, S). Fertigungsort: nicht belegt; Eigenfertigung nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Solingen, NRW)]</t>
+          <t>Lindgesfeld 8h, 42653 Solingen (Telefonbuch-Snippet, S). Fertigungsort: nicht belegt; Eigenfertigung nicht belegt.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -4515,12 +4559,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Sitz laut Verzeichnissen Siemensstraße 1, 63263 Neu-Isenburg (S, Verzeichnis). Fertigung in DE/AT/NL nicht belegt; Konzern KEYENCE Corp., Osaka.  [Gebiet: Rest Deutschland+Niederlande (Neu-Isenburg, …]</t>
+          <t>Sitz laut Verzeichnissen Siemensstraße 1, 63263 Neu-Isenburg (S, Verzeichnis). Fertigung in DE/AT/NL nicht belegt; Konzern KEYENCE Corp., Osaka.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Niedrig, Stufe S. Begründung: Suchergebnisse (Wikipedia-Spiegel, Firmenprofil) beschreiben Keyence als Entwickler ohne eigene Fertigung (Auftragsfertiger); GlobalData nennt Fertigungs- und Lagerstandorte in Asien, Europa, Amerika ohne Ort. Stellenanzeigen Neu-Isenburg: nur Vertrieb/Produktmanagement (S), keine Montage. …</t>
+          <t>Niedrig, Stufe S. Begründung: Suchergebnisse (Wikipedia-Spiegel, Firmenprofil) beschreiben Keyence als Entwickler ohne eigene Fertigung (Auftragsfertiger); GlobalData nennt Fertigungs- und Lagerstandorte in Asien, Europa, Amerika ohne Ort. Stellenanzeigen Neu-Isenburg: nur Vertrieb/Produktmanagement (S), keine Montage …</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -4575,7 +4619,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Willstätter Strasse 95, 90449 Nürnberg (S, Impressum-Snippet). Rolle des Standorts: Vertrieb/Service, ca. 25 Beschäftigte (Bayern International, S). Gruppenwerke: Komax SLE Grafenau, Schleuniger Haan (laut Triage), Schließungen Wiedensahl, Jettingen, Sömmerda …  [Gebiet: Bayern (Nürnberg)]</t>
+          <t>Willstätter Strasse 95, 90449 Nürnberg (S, Impressum-Snippet). Rolle des Standorts: Vertrieb/Service, ca. 25 Beschäftigte (Bayern International, S). Gruppenwerke: Komax SLE Grafenau, Schleuniger Haan (laut Triage), Schließungen Wiedensahl, Jettingen, Sömmerda …</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -4600,7 +4644,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>(a) Vertreibt oder fertigt die Komax Deutschland GmbH Nürnberg Dosier-/Vergusssysteme (Giebler, Wirth, 2-K-DOS)? Wo nachsehen: komaxgroup.com/de Produktseite "Dichten, Kleben, Vergießen" im Browser lesen, Ansprechpartnerseite Nürnberg, Impressum. Ist es belegt, ist es Rot nach E1 mit Quelle. (b) Wird in Nürnberg montiert (Stellenanzeigen Nürnberg: Montage, Produktion)? Falls nein und kein Dosiergeschäft: Rot nach E2/E3 nur mit V. (c) Gehören Schleuniger (Haan) und Komax SLE (Grafenau) zur selben Einheit? Aktion: …</t>
+          <t>(a) Vertreibt oder fertigt die Komax Deutschland GmbH Nürnberg Dosier-/Vergusssysteme (Giebler, Wirth, 2-K-DOS)? Wo nachsehen: komaxgroup.com/de Produktseite "Dichten, Kleben, Vergießen" im Browser lesen, Ansprechpartnerseite Nürnberg, Impressum. Ist es belegt, ist es Rot nach E1 mit Quelle. (b) Wird in Nürnberg montiert (Stellenanzeigen Nürnberg: Montage, Produktion)? Falls nein und kein Dosiergeschäft: Rot nach E2/E3 nur mit V. (c) Gehören Schleuniger (Haan) und Komax SLE (Grafenau) zur selben Einheit? Aktion …</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
@@ -4635,7 +4679,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Hoher Weg 13, 46325 Borken (Register-Aggregator, S). Teil der LB GmbH, Bocholt (S). Schaltschrankbau/Anlagenbau am Sitz laut Eigenprofil (S).  [Gebiet: Rest Deutschland+Niederlande (Borken-Weseke, NRW)]</t>
+          <t>Hoher Weg 13, 46325 Borken (Register-Aggregator, S). Teil der LB GmbH, Bocholt (S). Schaltschrankbau/Anlagenbau am Sitz laut Eigenprofil (S).</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -4695,7 +4739,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Im Stockacker 7, 78194 Immendingen (openPR, S). Produktion der Muttergesellschaft LASIT S.p.A. in Italien (Torre Annunziata/Vico Equense, Triage/openPR, S). Fertigung in Immendingen nicht belegt.  [Gebiet: Baden-Württemberg (Immendingen)]</t>
+          <t>Im Stockacker 7, 78194 Immendingen (openPR, S). Produktion der Muttergesellschaft LASIT S.p.A. in Italien (Torre Annunziata/Vico Equense, Triage/openPR, S). Fertigung in Immendingen nicht belegt.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -4755,7 +4799,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Sitz Essen, Büro Burgoberbach seit 2024; Mutter NTI AG, Spreitenbach (CH), produziert laut Triage in CH und SK. Das Unternehmen beschreibt Burgoberbach als Vertriebsbüro, nicht als Produktionsstandort (S).  [Gebiet: Rest Deutschland+Niederlande (Sitz Essen); Büro …]</t>
+          <t>Sitz Essen, Büro Burgoberbach seit 2024; Mutter NTI AG, Spreitenbach (CH), produziert laut Triage in CH und SK. Das Unternehmen beschreibt Burgoberbach als Vertriebsbüro, nicht als Produktionsstandort (S).</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -4815,7 +4859,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Im Ermlisgrund 30, Waldbronn (Triage, PDF-Quelle nicht gelesen, S). Konzernsitz Bergamo (IT). Fertigung Waldbronn: nicht belegt, Vertriebsniederlassung vermutet (Triage).  [Gebiet: Baden-Württemberg (Waldbronn, laut Triage)]</t>
+          <t>Im Ermlisgrund 30, Waldbronn (Triage, PDF-Quelle nicht gelesen, S). Konzernsitz Bergamo (IT). Fertigung Waldbronn: nicht belegt, Vertriebsniederlassung vermutet (Triage).</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -4875,7 +4919,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Meschede, PLZ 59872 laut Messeliste (aaa_duesseldorf_2026.csv); Fertigungsort unbekannt.  [Gebiet: Rest Deutschland+Niederlande (Meschede laut …]</t>
+          <t>Meschede, PLZ 59872 laut Messeliste (aaa_duesseldorf_2026.csv); Fertigungsort unbekannt.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -4935,7 +4979,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Wernau (Triage, laut DMG-MORI-Standortseite, S). Ob dort gefertigt oder nur vertrieben wird: nicht eindeutig (Triage).  [Gebiet: Baden-Württemberg (Wernau)]</t>
+          <t>Wernau (Triage, laut DMG-MORI-Standortseite, S). Ob dort gefertigt oder nur vertrieben wird: nicht eindeutig (Triage).</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -4995,7 +5039,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Winnettener Str. 6, 91550 Dinkelsbühl (Triage, Quelle Messe-Ausstellerseite, S). Fertigung am Sitz laut Eigenangabe "developed and manufactured in Germany" (Ausstellertext, S).  [Gebiet: Bayern (Dinkelsbühl)]</t>
+          <t>Winnettener Str. 6, 91550 Dinkelsbühl (Triage, Quelle Messe-Ausstellerseite, S). Fertigung am Sitz laut Eigenangabe "developed and manufactured in Germany" (Ausstellertext, S).</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -5015,7 +5059,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>unklar. crm_abgleich.py "MB connect line GmbH" und "MB connectline": kein Treffer. Nur das Kürzel "MB" liefert IDENTISCH (bekannte_firmen_DE-AT-NL.txt Zeile 1563, "MB [DE]", ohne Ort). Kürzel kann dieselbe Firma sein (Lehre 13), Zuordnung nicht möglich. …</t>
+          <t>unklar. crm_abgleich.py "MB connect line GmbH" und "MB connectline": kein Treffer. Nur das Kürzel "MB" liefert IDENTISCH (bekannte_firmen_DE-AT-NL.txt Zeile 1563, "MB [DE]", ohne Ort). Kürzel kann dieselbe Firma sein (Lehre 13), Zuordnung nicht möglich …</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -5055,7 +5099,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Waldkraiburg, Daimlerstraße 47, 84467 (S, Bayern-International-Eintrag). Eigenfertigung nicht belegt.  [Gebiet: Bayern (Waldkraiburg)]</t>
+          <t>Waldkraiburg, Daimlerstraße 47, 84467 (S, Bayern-International-Eintrag). Eigenfertigung nicht belegt.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -5115,7 +5159,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Steinfurt laut CSV-Vorgabe; keine Quelle gefunden. Fertigung unbekannt.  [Gebiet: Rest Deutschland+Niederlande (Steinfurt, laut …]</t>
+          <t>Steinfurt laut CSV-Vorgabe; keine Quelle gefunden. Fertigung unbekannt.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -5175,7 +5219,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Im Tal 2, 78176 Blumberg (S, Händlerlisting). Produktion am Sitz: Stellenanzeigen Spritzguss (Prozessoptimierer, Verfahrensmechaniker) bei Metz Connect Blumberg (S, Suchtreffer, nicht gelesen). Kooperation mit ESCHA (Halver) zu Entwicklung und Produktion von …  [Gebiet: Baden-Württemberg (Blumberg)]</t>
+          <t>Im Tal 2, 78176 Blumberg (S, Händlerlisting). Produktion am Sitz: Stellenanzeigen Spritzguss (Prozessoptimierer, Verfahrensmechaniker) bei Metz Connect Blumberg (S, Suchtreffer, nicht gelesen). Kooperation mit ESCHA (Halver) zu Entwicklung und Produktion von …</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -5185,7 +5229,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Mittel, Stufe A. Einzelbewertung: konfektionierte M12/LWL-Kabel Mittel (A; Konfektion durch Metz nicht belegt, Produkte teils feldkonfektionierbar), IP67-Steckverbinder/Durchführungen Mittel (A, Dichtungen), Klemmen/RJ45 Niedrig (A), Netzwerkkomponenten mit Elektronik Mittel (A). Triage nennt "Hoch" für konfektionierte Kabel; …</t>
+          <t>Mittel, Stufe A. Einzelbewertung: konfektionierte M12/LWL-Kabel Mittel (A; Konfektion durch Metz nicht belegt, Produkte teils feldkonfektionierbar), IP67-Steckverbinder/Durchführungen Mittel (A, Dichtungen), Klemmen/RJ45 Niedrig (A), Netzwerkkomponenten mit Elektronik Mittel (A). Triage nennt "Hoch" für konfektionierte Kabel …</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -5235,7 +5279,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Großmaischeid, Westerwald (S, Presse/it-daily-Snippet); Adresse nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Großmaischeid, …]</t>
+          <t>Großmaischeid, Westerwald (S, Presse/it-daily-Snippet); Adresse nicht belegt.</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -5295,7 +5339,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>MiniTec Allee 1, 66901 Schönenberg-Kübelberg, Headquarter mit 12.000 m² Produktionsfläche und 3.000 m² Büros (S, Firmenbroschüre im Suchsnippet). Gruppe mit ca. 11 Standorten (DE, FR, USA, UK, ES, SK, SI, CN), ca. 420 Mitarbeitende (S). Fertigende Einheit für …  [Gebiet: Rest Deutschland+Niederlande …]</t>
+          <t>MiniTec Allee 1, 66901 Schönenberg-Kübelberg, Headquarter mit 12.000 m² Produktionsfläche und 3.000 m² Büros (S, Firmenbroschüre im Suchsnippet). Gruppe mit ca. 11 Standorten (DE, FR, USA, UK, ES, SK, SI, CN), ca. 420 Mitarbeitende (S). Fertigende Einheit für …</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -5355,7 +5399,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Wuppertal (S, Messeprofil); Adresse nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Wuppertal, NRW)]</t>
+          <t>Wuppertal (S, Messeprofil); Adresse nicht belegt.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -5415,7 +5459,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Verzeichnisse (directindustry, yumda, Firmenbroschüre) nennen In der Wanne 55, 89075 Ulm (S); St. Ingbert (CSV-Vorgabe) ist in keiner Suchquelle belegt. Fertigung am Sitz Ulm: "entwickelt und produziert seit 2003" (S, Profiltext).  [Gebiet: Baden-Württemberg (Ulm laut Verzeichnissen) bzw. …]</t>
+          <t>Verzeichnisse (directindustry, yumda, Firmenbroschüre) nennen In der Wanne 55, 89075 Ulm (S); St. Ingbert (CSV-Vorgabe) ist in keiner Suchquelle belegt. Fertigung am Sitz Ulm: "entwickelt und produziert seit 2003" (S, Profiltext).</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -5475,7 +5519,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Vorgabe Lisle IL (USA). Deutschland: Molex Deutschland GmbH, Otto-Hahn-Straße 1b, 69190 Walldorf (S, elektroniknet.de-Anbieterkompass); Ettlingen nur als Händleradresse (Grashofstr. 17) gefunden, KEIN Beleg für ein Werk (S). Werke in Deutschland (Ettlingen, …  [Gebiet: außerhalb (Vorgabe-Sitz USA); deutsche Einheiten …]</t>
+          <t>Vorgabe Lisle IL (USA). Deutschland: Molex Deutschland GmbH, Otto-Hahn-Straße 1b, 69190 Walldorf (S, elektroniknet.de-Anbieterkompass); Ettlingen nur als Händleradresse (Grashofstr. 17) gefunden, KEIN Beleg für ein Werk (S). Werke in Deutschland (Ettlingen …</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -5535,7 +5579,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Im Fange 1, 49356 Diepholz (Verzeichniseintrag, S). Fertigungsort nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Diepholz, …]</t>
+          <t>Im Fange 1, 49356 Diepholz (Verzeichniseintrag, S). Fertigungsort nicht belegt.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -5595,7 +5639,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Achim laut Messeliste; in den Suchergebnissen nicht bestätigt (S). Fertigungsort nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Achim, …]</t>
+          <t>Achim laut Messeliste; in den Suchergebnissen nicht bestätigt (S). Fertigungsort nicht belegt.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -5655,7 +5699,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Bischofstraße 99, 47809 Krefeld (Verzeichnis, S); Krefeld = europäische Zentrale und Logistikzentrum, Vertrieb/Service (S). Werke der Gruppe in Tschechien (Katalog, S). Fertigung in Krefeld nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Krefeld, NRW)]</t>
+          <t>Bischofstraße 99, 47809 Krefeld (Verzeichnis, S); Krefeld = europäische Zentrale und Logistikzentrum, Vertrieb/Service (S). Werke der Gruppe in Tschechien (Katalog, S). Fertigung in Krefeld nicht belegt.</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -5715,7 +5759,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Wegberg laut Messeliste; die Suche fand keine Firmenseite, kein Impressum, keine Adresse (S). Fertigungsort nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Wegberg, NRW, laut …]</t>
+          <t>Wegberg laut Messeliste; die Suche fand keine Firmenseite, kein Impressum, keine Adresse (S). Fertigungsort nicht belegt.</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -5775,7 +5819,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Edisonstraße 7, 60388 Frankfurt (Stellenanzeige, Datenschutzhinweis, S). Kabelkonfektion laut Stellenanzeige in der Abteilung am Standort (S).  [Gebiet: Rest Deutschland+Niederlande (Frankfurt am Main, …]</t>
+          <t>Edisonstraße 7, 60388 Frankfurt (Stellenanzeige, Datenschutzhinweis, S). Kabelkonfektion laut Stellenanzeige in der Abteilung am Standort (S).</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -5795,7 +5839,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>neu mit Hinweis. crm_abgleich.py "NIES electronic gmbh": nur AEHNLICH 0.90 zu "CiS Electronic GmbH [DE]" (bekannte_firmen Zeile 413); Kern-Name verschieden ("nies electronic" vs. "cis electronic"), laut Triage erkennbar andere Firma. …</t>
+          <t>neu mit Hinweis. crm_abgleich.py "NIES electronic gmbh": nur AEHNLICH 0.90 zu "CiS Electronic GmbH [DE]" (bekannte_firmen Zeile 413); Kern-Name verschieden ("nies electronic" vs. "cis electronic"), laut Triage erkennbar andere Firma …</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -5835,7 +5879,7 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Alpen, Bruckstraße 93 (RS-Online-Herstellerangabe, S); ein Branchenverzeichnis nennt Stuttgarter Str. 120, Fellbach (S). Fertigung in beiden nicht belegt. Eine RS-Produktseite (Norgren V61 Magnetventil) nennt Herkunftsland CZ (S), also mindestens teilweise …  [Gebiet: Rest Deutschland+Niederlande (Alpen, NRW laut …]</t>
+          <t>Alpen, Bruckstraße 93 (RS-Online-Herstellerangabe, S); ein Branchenverzeichnis nennt Stuttgarter Str. 120, Fellbach (S). Fertigung in beiden nicht belegt. Eine RS-Produktseite (Norgren V61 Magnetventil) nennt Herkunftsland CZ (S), also mindestens teilweise …</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -5860,7 +5904,7 @@
       </c>
       <c r="J91" s="2" t="inlineStr">
         <is>
-          <t>(1) Jey: Ist "IMI [DE]" (Zeile 1127) die IMI plc / IMI Precision Engineering bzw. eine Schwester (Norgren, Buschjost, Herion), oder eine andere Firma? Wo nachsehen: CRM-Datensatz (Adresse, Ansprechpartner, Kundennummer), Handelsregister der Norgren GmbH (Amtsgericht Kleve) und von "IMI" (falls GmbH). (2) Wird in Alpen gefertigt (Magnetventile, Spulen, Baugruppen) und welche Einheit (Norgren/Herion/Buschjost) fertigt wo? Wo nachsehen: Standortseite IMI Precision Engineering, Impressum norgren.com/de, …</t>
+          <t>(1) Jey: Ist "IMI [DE]" (Zeile 1127) die IMI plc / IMI Precision Engineering bzw. eine Schwester (Norgren, Buschjost, Herion), oder eine andere Firma? Wo nachsehen: CRM-Datensatz (Adresse, Ansprechpartner, Kundennummer), Handelsregister der Norgren GmbH (Amtsgericht Kleve) und von "IMI" (falls GmbH). (2) Wird in Alpen gefertigt (Magnetventile, Spulen, Baugruppen) und welche Einheit (Norgren/Herion/Buschjost) fertigt wo? Wo nachsehen: Standortseite IMI Precision Engineering, Impressum norgren.com/de …</t>
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr">
@@ -5895,7 +5939,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Soest = Büro (DACH/Benelux) (Verzeichnis, S). Hauptsitz OnRobot A/S, Teglværksvej 47H, Odense, Dänemark (S). Fertigungsort der Greifer in keiner Quelle genannt.  [Gebiet: Rest Deutschland+Niederlande (Soest, NRW laut …]</t>
+          <t>Soest = Büro (DACH/Benelux) (Verzeichnis, S). Hauptsitz OnRobot A/S, Teglværksvej 47H, Odense, Dänemark (S). Fertigungsort der Greifer in keiner Quelle genannt.</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -5955,7 +5999,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Freiburg im Breisgau (Verzeichnis, S); Profil: "alle unsere Lösungen am Standort Freiburg entwickelt und hergestellt" (Firmenprofil, Suchzusammenfassung, S).  [Gebiet: Baden-Württemberg (Freiburg im Breisgau)]</t>
+          <t>Freiburg im Breisgau (Verzeichnis, S); Profil: "alle unsere Lösungen am Standort Freiburg entwickelt und hergestellt" (Firmenprofil, Suchzusammenfassung, S).</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -6015,7 +6059,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Solingen (42653) laut Messeliste, Stufe A/S; laut Triage "Sitz unbestätigt". Fertigende Einheit nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Solingen, NRW, laut …]</t>
+          <t>Solingen (42653) laut Messeliste, Stufe A/S; laut Triage "Sitz unbestätigt". Fertigende Einheit nicht belegt.</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -6046,7 +6090,7 @@
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>Identität/Sitz nur aus Messeliste, keine Website</t>
+          <t>ja</t>
         </is>
       </c>
     </row>
@@ -6071,7 +6115,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Sitz Friedrichstraße, Stuttgart (S, Suchsnippet peakboard.com/en/imprint; Triage: Friedrichstr. 13). Fertigungsort der Hardware: nicht belegt.  [Gebiet: Baden-Württemberg (Stuttgart)]</t>
+          <t>Sitz Friedrichstraße, Stuttgart (S, Suchsnippet peakboard.com/en/imprint; Triage: Friedrichstr. 13). Fertigungsort der Hardware: nicht belegt.</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -6102,7 +6146,7 @@
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>Fertigung der Box unbekannt, E2 (Software) nicht V-belegt</t>
+          <t>nein</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6171,7 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Hauptsitz Hamburg, Werner-Witt-Straße 1 (S, Suchsnippet pfannenberg.com). Produktionsstandorte "in Germany, Italy, the United States and China" (S, Eigenangabe pfannenberg.com global-set-up); ob Hamburg selbst produziert und welche Produkte dort entstehen, …  [Gebiet: Rest Deutschland+Niederlande (Hamburg; Messeliste …]</t>
+          <t>Hauptsitz Hamburg, Werner-Witt-Straße 1 (S, Suchsnippet pfannenberg.com). Produktionsstandorte "in Germany, Italy, the United States and China" (S, Eigenangabe pfannenberg.com global-set-up); ob Hamburg selbst produziert und welche Produkte dort entstehen …</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -6158,7 +6202,7 @@
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>Vorgabe Wülfrath nicht belegt; Hamburg gefunden</t>
+          <t>ja</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6227,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Sitz Ostfildern (73760); "Neben dem Werk am Stammsitz in Ostfildern produziert Pilz auch in Betschdorf (Frankreich)" und Jintan (China) (S, Suchsnippet industrial-production.de). Fertigende Einheit für DE: Ostfildern.  [Gebiet: Baden-Württemberg (Ostfildern)]</t>
+          <t>Sitz Ostfildern (73760); "Neben dem Werk am Stammsitz in Ostfildern produziert Pilz auch in Betschdorf (Frankreich)" und Jintan (China) (S, Suchsnippet industrial-production.de). Fertigende Einheit für DE: Ostfildern.</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -6214,7 +6258,7 @@
       </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t>Konzern/mehrere Werke, V für Ostfildern fehlt</t>
+          <t>ja</t>
         </is>
       </c>
     </row>
@@ -6239,7 +6283,7 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Lüdenscheid (58513), "owner-operated business ... 40 employees at the Luedenscheid site" (S, Messe-/Firmenprofil-Snippet). Fertigung der Hubtüren am Standort laut Eigenangabe (S).  [Gebiet: Rest Deutschland+Niederlande (Lüdenscheid, NRW)]</t>
+          <t>Lüdenscheid (58513), "owner-operated business ... 40 employees at the Luedenscheid site" (S, Messe-/Firmenprofil-Snippet). Fertigung der Hubtüren am Standort laut Eigenangabe (S).</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -6270,7 +6314,7 @@
       </c>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t>Händler-Mischform, Eigenfertigung nur Eigenangabe (S)</t>
+          <t>nein</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6339,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Zeppelinstraße 11, 78256 Steißlingen (S, embedded-world.de-Aussteller-Listing und MECSPE-Profil); "manufacturing sites in Germany and Taiwan / China" (S, Profil-Snippet). Welche Produkte in Steißlingen entstehen, ist nicht belegt.  [Gebiet: Baden-Württemberg (Steißlingen)]</t>
+          <t>Zeppelinstraße 11, 78256 Steißlingen (S, embedded-world.de-Aussteller-Listing und MECSPE-Profil); "manufacturing sites in Germany and Taiwan / China" (S, Profil-Snippet). Welche Produkte in Steißlingen entstehen, ist nicht belegt.</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -6326,7 +6370,7 @@
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>Vorgabe Wülfrath nicht belegt; Steißlingen gefunden</t>
+          <t>ja</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6395,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Köln (50676) laut Messeliste (A/S); im Suchlauf nicht bestätigt (Messelisting nennt keine Stadt). Fertigungsort unbekannt.  [Gebiet: Rest Deutschland+Niederlande (Köln laut …]</t>
+          <t>Köln (50676) laut Messeliste (A/S); im Suchlauf nicht bestätigt (Messelisting nennt keine Stadt). Fertigungsort unbekannt.</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -6382,7 +6426,7 @@
       </c>
       <c r="L100" s="2" t="inlineStr">
         <is>
-          <t>Identität/Standort nicht belegt, Patent-/Böhrer-Hinweis</t>
+          <t>ja</t>
         </is>
       </c>
     </row>
@@ -6407,7 +6451,7 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Wörth am Main (63939) Hauptsitz, neues Gebäude "mit mehr Platz für Produktion und Verwaltung" (S, Suchsnippet); Töchter USA, China, Italien, Frankreich, Slowakei (S). Ein Verzeichnis nennt abweichend Klingenberg (PLZ 63929), Widerspruch ungeklärt.  [Gebiet: Bayern (Wörth am Main)]</t>
+          <t>Wörth am Main (63939) Hauptsitz, neues Gebäude "mit mehr Platz für Produktion und Verwaltung" (S, Suchsnippet); Töchter USA, China, Italien, Frankreich, Slowakei (S). Ein Verzeichnis nennt abweichend Klingenberg (PLZ 63929), Widerspruch ungeklärt.</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -6438,7 +6482,7 @@
       </c>
       <c r="L101" s="2" t="inlineStr">
         <is>
-          <t>Gruppe mit Auslandstöchtern, V für Wörth fehlt</t>
+          <t>ja</t>
         </is>
       </c>
     </row>
@@ -6463,7 +6507,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Duisburg (Spin-off Uni Duisburg-Essen, S: uni-due.de, bouncewatch/Verzeichnis, KEBA-Success-Story "Duisburg start-up"). Fertigungsort: nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Duisburg, NRW; …]</t>
+          <t>Duisburg (Spin-off Uni Duisburg-Essen, S: uni-due.de, bouncewatch/Verzeichnis, KEBA-Success-Story "Duisburg start-up"). Fertigungsort: nicht belegt.</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -6494,7 +6538,7 @@
       </c>
       <c r="L102" s="2" t="inlineStr">
         <is>
-          <t>Vorgabe Hoppstädten-Weiersbach nicht belegt; Duisburg gefunden</t>
+          <t>ja</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6563,7 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Kaiserslautern (67663) laut Messeliste; Firma per Suche nicht auffindbar. Fertigungsort unbekannt.  [Gebiet: Rest Deutschland+Niederlande (Kaiserslautern laut …]</t>
+          <t>Kaiserslautern (67663) laut Messeliste; Firma per Suche nicht auffindbar. Fertigungsort unbekannt.</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -6550,7 +6594,7 @@
       </c>
       <c r="L103" s="2" t="inlineStr">
         <is>
-          <t>Firma nicht auffindbar</t>
+          <t>ja</t>
         </is>
       </c>
     </row>
@@ -6575,7 +6619,7 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Robert-Bosch-Str. 3, 51674 Wiehl-Bomig; "own developing, processing and manufacturing factory in Wiehl" (S). Mehrheit bei DELFINGEN (FR) seit 2023 (Triage, S), Gruppe ca. 3.800 MA, 40 Standorte (Stellenanzeige, S).  [Gebiet: Rest Deutschland+Niederlande (Wiehl, NRW)]</t>
+          <t>Robert-Bosch-Str. 3, 51674 Wiehl-Bomig; "own developing, processing and manufacturing factory in Wiehl" (S). Mehrheit bei DELFINGEN (FR) seit 2023 (Triage, S), Gruppe ca. 3.800 MA, 40 Standorte (Stellenanzeige, S).</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -6635,7 +6679,7 @@
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Potsdamer Str. 9, 32423 Minden (Stammsitz, S); "rund 210 [MA] am Stammsitz in Minden" (S). Fertigung in eigenen Hallen in Minden (Triage, S). Tochter der Phoenix Mecano AG (CH), weitere RK-Standorte nicht geprüft.  [Gebiet: Rest Deutschland+Niederlande (Minden, NRW)]</t>
+          <t>Potsdamer Str. 9, 32423 Minden (Stammsitz, S); "rund 210 [MA] am Stammsitz in Minden" (S). Fertigung in eigenen Hallen in Minden (Triage, S). Tochter der Phoenix Mecano AG (CH), weitere RK-Standorte nicht geprüft.</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -6695,7 +6739,7 @@
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>Max-Planck-Str. 4, Aschheim (CB Insights-Snippet, S); Fertigungsort NICHT belegt.  [Gebiet: Bayern (Aschheim bei München)]</t>
+          <t>Max-Planck-Str. 4, Aschheim (CB Insights-Snippet, S); Fertigungsort NICHT belegt.</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -6755,7 +6799,7 @@
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Philipp-Reis-Str. 23, 45659 Recklinghausen (Verzeichnis-Snippet, S); Sondermaschinenbau/Zellenbau dort (S).  [Gebiet: Rest Deutschland+Niederlande (Recklinghausen, NRW)]</t>
+          <t>Philipp-Reis-Str. 23, 45659 Recklinghausen (Verzeichnis-Snippet, S); Sondermaschinenbau/Zellenbau dort (S).</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
@@ -6815,7 +6859,7 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Hagen (Messe-/Verzeichnis-Snippets). Anschrift widersprüchlich: Triage Pappelstr. 28A, 58099 vs. Vorgabe PLZ 58093; das Triage-Verzeichnis (11880, Suchbegriff "Sundern") ist als Quelle unsicher. Fertigung: Messeprofil sagt "developed and manufactured" …  [Gebiet: Rest Deutschland+Niederlande (Hagen, NRW)]</t>
+          <t>Hagen (Messe-/Verzeichnis-Snippets). Anschrift widersprüchlich: Triage Pappelstr. 28A, 58099 vs. Vorgabe PLZ 58093; das Triage-Verzeichnis (11880, Suchbegriff "Sundern") ist als Quelle unsicher. Fertigung: Messeprofil sagt "developed and manufactured" …</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
@@ -6875,7 +6919,7 @@
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Max-Planck-Straße 20, 78549 Spaichingen (Messe-/Verzeichnis-Snippets, S). Fertigung: nicht belegt.  [Gebiet: Baden-Württemberg (Spaichingen)]</t>
+          <t>Max-Planck-Straße 20, 78549 Spaichingen (Messe-/Verzeichnis-Snippets, S). Fertigung: nicht belegt.</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -6935,7 +6979,7 @@
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Am Bruch 21-23, 42857 Remscheid (Verzeichnis, S); ehemals SIC-Wostor Markiersysteme GmbH (Pressemeldung 2014, S). Fertigung in Remscheid NICHT bestätigt: Suche fand nur Adresse; Nill + Ritz (Markgröningen, ca. 25 MA) baut kundenspezifische Markierstationen …  [Gebiet: Rest Deutschland+Niederlande (Remscheid, NRW); …]</t>
+          <t>Am Bruch 21-23, 42857 Remscheid (Verzeichnis, S); ehemals SIC-Wostor Markiersysteme GmbH (Pressemeldung 2014, S). Fertigung in Remscheid NICHT bestätigt: Suche fand nur Adresse; Nill + Ritz (Markgröningen, ca. 25 MA) baut kundenspezifische Markierstationen …</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -6995,7 +7039,7 @@
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>Mahdenstraße 3, 72768 Reutlingen (S, Verzeichnis). Fertigung am Sitz: Verzeichnis nennt "Entwicklung und Produktion von Industrie-PCs" (S). Töchter CH, AT; Seit 07/2025 ICP Deutschland Teil von Spectra (Triage, A). Fertigende Einheit: Reutlingen (nicht …  [Gebiet: Baden-Württemberg (Reutlingen)]</t>
+          <t>Mahdenstraße 3, 72768 Reutlingen (S, Verzeichnis). Fertigung am Sitz: Verzeichnis nennt "Entwicklung und Produktion von Industrie-PCs" (S). Töchter CH, AT; Seit 07/2025 ICP Deutschland Teil von Spectra (Triage, A). Fertigende Einheit: Reutlingen (nicht …</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
@@ -7055,7 +7099,7 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>Attnang-Puchheim, Salzburger Straße 52 (Triage, WKO-Eintrag, A). Fertigung der Gruppe: STIWA Manufacturing Austria in Gampern, Technologiepark 10 (S). Fertigende Einheit für Produkte also Gampern, nicht belegt für "AMS".  [Gebiet: Österreich (Attnang-Puchheim; Gruppe auch Gampern)]</t>
+          <t>Attnang-Puchheim, Salzburger Straße 52 (Triage, WKO-Eintrag, A). Fertigung der Gruppe: STIWA Manufacturing Austria in Gampern, Technologiepark 10 (S). Fertigende Einheit für Produkte also Gampern, nicht belegt für "AMS".</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -7115,7 +7159,7 @@
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>Attnang-Puchheim (Triage; Firmenbuch evi.gv.at/f/295396g aus Triage, nicht geprüft). Fertigung: Eigene Montageanlagen/Automationssysteme (S).  [Gebiet: Österreich (Attnang-Puchheim)]</t>
+          <t>Attnang-Puchheim (Triage; Firmenbuch evi.gv.at/f/295396g aus Triage, nicht geprüft). Fertigung: Eigene Montageanlagen/Automationssysteme (S).</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
@@ -7175,7 +7219,7 @@
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>Golling an der Salzach, Holzerfeld 397 (Triage, aaa-Messeseite S). Die Websuche bestätigte Golling/Salzburg NICHT (keine Adressangabe in den Treffern). Fertigung: nicht belegt.  [Gebiet: Österreich (Golling an der Salzach laut Liste)]</t>
+          <t>Golling an der Salzach, Holzerfeld 397 (Triage, aaa-Messeseite S). Die Websuche bestätigte Golling/Salzburg NICHT (keine Adressangabe in den Treffern). Fertigung: nicht belegt.</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
@@ -7235,7 +7279,7 @@
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>Flurweg 12, 84069 Schierling (Hauptsitz laut Presse 2018, S); Vertriebsstandort Coesfeld. Fertigung in Schierling: NICHT belegt (Suche: "Ob Handsender in Schierling gefertigt werden, geht aus diesen Quellen nicht hervor"). Gruppe: schwedische Tele Radio …  [Gebiet: Bayern (Schierling)]</t>
+          <t>Flurweg 12, 84069 Schierling (Hauptsitz laut Presse 2018, S); Vertriebsstandort Coesfeld. Fertigung in Schierling: NICHT belegt (Suche: "Ob Handsender in Schierling gefertigt werden, geht aus diesen Quellen nicht hervor"). Gruppe: schwedische Tele Radio …</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
@@ -7295,7 +7339,7 @@
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>Joseph-Gänsler-Straße 10, 86609 Donauwörth (Hauptsitz und Logistikzentrum, S). Eigene Fertigung: nicht belegt.  [Gebiet: Bayern (Donauwörth)]</t>
+          <t>Joseph-Gänsler-Straße 10, 86609 Donauwörth (Hauptsitz und Logistikzentrum, S). Eigene Fertigung: nicht belegt.</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
@@ -7355,7 +7399,7 @@
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>Oberdörnen 74, 42283 Wuppertal (S, Verzeichnis). Gegründet 2005 von Hartmut Linde (Cylex, S). Eigenfertigung: NICHT belegt (Suche: "None of the results describe production at the Oberdörnen site").  [Gebiet: Rest Deutschland+Niederlande (Wuppertal, NRW)]</t>
+          <t>Oberdörnen 74, 42283 Wuppertal (S, Verzeichnis). Gegründet 2005 von Hartmut Linde (Cylex, S). Eigenfertigung: NICHT belegt (Suche: "None of the results describe production at the Oberdörnen site").</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
@@ -7415,7 +7459,7 @@
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>Trossingen (aaa-Messeseite, S); Division Unidor evtl. Pforzheim (Triage, per Websuche nicht bestätigt: "no Pforzheim reference"). Fertigung am Sitz: nicht belegt; Tochter der TR-Electronic GmbH, Trossingen (Hauptsitz, 350+ Mitarbeiter, S).  [Gebiet: Baden-Württemberg (Trossingen)]</t>
+          <t>Trossingen (aaa-Messeseite, S); Division Unidor evtl. Pforzheim (Triage, per Websuche nicht bestätigt: "no Pforzheim reference"). Fertigung am Sitz: nicht belegt; Tochter der TR-Electronic GmbH, Trossingen (Hauptsitz, 350+ Mitarbeiter, S).</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
@@ -7475,7 +7519,7 @@
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>Esslingen (Liste); Indeed-Stellen in Esslingen (Technischer Support, NPI-Engineering, Vertrieb, S) deuten auf deutsche Niederlassung hin, keine Fertigung. Stammhaus Unitronics (1989) (R"G) Ltd., Israel, "design, development, production, marketing" von SPS …  [Gebiet: Baden-Württemberg (Esslingen laut Liste)]</t>
+          <t>Esslingen (Liste); Indeed-Stellen in Esslingen (Technischer Support, NPI-Engineering, Vertrieb, S) deuten auf deutsche Niederlassung hin, keine Fertigung. Stammhaus Unitronics (1989) (R"G) Ltd., Israel, "design, development, production, marketing" von SPS …</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
@@ -7535,7 +7579,7 @@
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>Schwerte laut Liste/Vorgabe (unverifiziert); Fertigung unbekannt.  [Gebiet: Rest Deutschland+Niederlande (Schwerte laut …]</t>
+          <t>Schwerte laut Liste/Vorgabe (unverifiziert); Fertigung unbekannt.</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -7580,10 +7624,14 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>W.E.S.T Elektronik GmbH (523) | prüfenswert</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="inlineStr"/>
+          <t>W.E.S.T Elektronik GmbH</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>523</t>
+        </is>
+      </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -7591,7 +7639,7 @@
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>laut Verzeichnis (S) W.E.St. Elektronik GmbH, Gewerbering 31, 41372 Niederkrüchten; Fertigungsort nicht belegt. Spaichingen laut Liste unbelegt (Schuhmacher Technologies &amp; Hydraulics GmbH nennt sich Generalvertretung von WEST, Adresse nicht erkennbar, S).  [Gebiet: Rest Deutschland+Niederlande (Niederkrüchten, NRW …]</t>
+          <t>laut Verzeichnis (S) W.E.St. Elektronik GmbH, Gewerbering 31, 41372 Niederkrüchten; Fertigungsort nicht belegt. Spaichingen laut Liste unbelegt (Schuhmacher Technologies &amp; Hydraulics GmbH nennt sich Generalvertretung von WEST, Adresse nicht erkennbar, S).</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
@@ -7636,10 +7684,14 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Wachendorff Prozesstechnik GmbH &amp; Co. KG (623) | interessant</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="inlineStr"/>
+          <t>Wachendorff Prozesstechnik GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>623</t>
+        </is>
+      </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -7647,7 +7699,7 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>Industriestr. 7, 65366 Geisenheim; laut Verzeichnis Management, Entwicklung, Lager und Produktion (S, automationindiaexpo.com, Wachendorff Automation GmbH &amp; Co. KG). Fertigende Einheit für Encoder: vermutlich Wachendorff Automation GmbH &amp; Co. KG (Gruppe), …  [Gebiet: Rest Deutschland+Niederlande (Geisenheim, Hessen)]</t>
+          <t>Industriestr. 7, 65366 Geisenheim; laut Verzeichnis Management, Entwicklung, Lager und Produktion (S, automationindiaexpo.com, Wachendorff Automation GmbH &amp; Co. KG). Fertigende Einheit für Encoder: vermutlich Wachendorff Automation GmbH &amp; Co. KG (Gruppe) …</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -7692,10 +7744,14 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>Wagner GmbH (435) | kein Fertiger</t>
-        </is>
-      </c>
-      <c r="C123" s="2" t="inlineStr"/>
+          <t>Wagner GmbH</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>435</t>
+        </is>
+      </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
           <t>GELB (Rot-Kandidat E2)</t>
@@ -7703,7 +7759,7 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>Robert-Bosch-Str. 35, Wülfrath (S, StepStone/Cylex). Keine Fertigung belegt.  [Gebiet: Rest Deutschland+Niederlande (Wülfrath, NRW)]</t>
+          <t>Robert-Bosch-Str. 35, Wülfrath (S, StepStone/Cylex). Keine Fertigung belegt.</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
@@ -7748,10 +7804,14 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Walter Rothermundt GmbH &amp; Co. KG (716) | unwahrscheinlich</t>
-        </is>
-      </c>
-      <c r="C124" s="2" t="inlineStr"/>
+          <t>Walter Rothermundt GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>716</t>
+        </is>
+      </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -7759,7 +7819,7 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>Mönchengladbach laut Liste (Stufe ?, keine Quelle zum Ort gefunden). Fertigungsort nicht belegt.  [Gebiet: Rest Deutschland+Niederlande (Mönchengladbach, …]</t>
+          <t>Mönchengladbach laut Liste (Stufe ?, keine Quelle zum Ort gefunden). Fertigungsort nicht belegt.</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -7804,10 +7864,14 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>WEG Germany GmbH (421) | prüfenswert</t>
-        </is>
-      </c>
-      <c r="C125" s="2" t="inlineStr"/>
+          <t>WEG Germany GmbH</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>421</t>
+        </is>
+      </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
           <t>GELB</t>
@@ -7815,12 +7879,12 @@
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>Industriegebiet Türnich 3, Röntgenstraße 36-38, 50169 Kerpen-Türnich (S, weg.net laut Suchzusammenfassung). Fertigende Einheit: Kerpen (Stellenanzeige Fertigungsmitarbeiter Antriebskomponenten, S), Balingen (Württembergische Elektromotoren, übernommen, …  [Gebiet: Rest Deutschland+Niederlande (Kerpen, NRW); …]</t>
+          <t>Industriegebiet Türnich 3, Röntgenstraße 36-38, 50169 Kerpen-Türnich (S, weg.net laut Suchzusammenfassung). Fertigende Einheit: Kerpen (Stellenanzeige Fertigungsmitarbeiter Antriebskomponenten, S), Balingen (Württembergische Elektromotoren, übernommen …</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>Mittel, Stufe S. Begründung: Konzern mit mehreren Werken (V nötig, nicht erreicht). Belege nur S: Stellenanzeige "Mechatroniker/Elektroniker als Fertigungsmitarbeiter für Antriebskomponenten" Kerpen (Aggregator-Snippet, undatiert), Übernahmemeldung Balingen 2014 mit "manufacturing plants in Balingen". Einheitenzuordnung offen: …</t>
+          <t>Mittel, Stufe S. Begründung: Konzern mit mehreren Werken (V nötig, nicht erreicht). Belege nur S: Stellenanzeige "Mechatroniker/Elektroniker als Fertigungsmitarbeiter für Antriebskomponenten" Kerpen (Aggregator-Snippet, undatiert), Übernahmemeldung Balingen 2014 mit "manufacturing plants in Balingen". Einheitenzuordnung offen …</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -7835,7 +7899,7 @@
       </c>
       <c r="I125" s="2" t="inlineStr">
         <is>
-          <t>unklar, CRM-Konzernbezug (Regel M). crm_abgleich.py "WEG Germany GmbH" und "WEG": kein Treffer. Aber: WEG hat laut Fachpresse (S) KATT Antriebstechnik (Homberg) übernommen ("Jetzt fünf Filialen in Deutschland: WEG übernimmt Katt Antriebstechnik", …</t>
+          <t>unklar, CRM-Konzernbezug (Regel M). crm_abgleich.py "WEG Germany GmbH" und "WEG": kein Treffer. Aber: WEG hat laut Fachpresse (S) KATT Antriebstechnik (Homberg) übernommen ("Jetzt fünf Filialen in Deutschland: WEG übernimmt Katt Antriebstechnik" …</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
@@ -7860,10 +7924,14 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Yaskawa Europe GmbH – Drives Motion Controls Division (630) | unwahrscheinlich</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr"/>
+          <t>Yaskawa Europe GmbH – Drives Motion Controls Division</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>630</t>
+        </is>
+      </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
           <t>GELB (Rot-Kandidat E3)</t>
@@ -7871,7 +7939,7 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>Sitz Hattersheim (Europazentrale, Bürogebäude mit Training Center und Innovation Center, kein Produktionsbetrieb belegt, S). Drive-Fertigung Europa: Cumbernauld (Schottland) und geplante Werke in Slowenien (Kočevje, Meldung 2018, Stand unbekannt); Roboterwerk …  [Gebiet: Rest Deutschland+Niederlande (Hattersheim, …]</t>
+          <t>Sitz Hattersheim (Europazentrale, Bürogebäude mit Training Center und Innovation Center, kein Produktionsbetrieb belegt, S). Drive-Fertigung Europa: Cumbernauld (Schottland) und geplante Werke in Slowenien (Kočevje, Meldung 2018, Stand unbekannt); Roboterwerk …</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
@@ -7931,7 +7999,7 @@
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>Bendstraße 50, 52066 Aachen (Impressum, S). Keine Fertigung belegt.  [Gebiet: Rest Deutschland+Niederlande (Aachen, NRW)]</t>
+          <t>Bendstraße 50, 52066 Aachen (Impressum, S). Keine Fertigung belegt.</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
@@ -7983,7 +8051,7 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>Schubertstraße 47, 78054 Villingen-Schwenningen (S, Betriebsanleitung). Gruppe mit Produktionsstandorten in Europa, Asien, USA (Pune, Charlotte laut Triage). Welche Produkte in Schwenningen entstehen: nicht belegt.  [Gebiet: Baden-Württemberg (Villingen-Schwenningen)]</t>
+          <t>Schubertstraße 47, 78054 Villingen-Schwenningen (S, Betriebsanleitung). Gruppe mit Produktionsstandorten in Europa, Asien, USA (Pune, Charlotte laut Triage). Welche Produkte in Schwenningen entstehen: nicht belegt.</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
@@ -8034,7 +8102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -8043,42 +8111,21 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Stand 2026-10-15, Messe all about automation Düsseldorf 2026 (aaa). Geprüft: 127 Firmen mit Tom v2 und Tina v2. Dazu 41 Aussteller bereits im CRM und 54 in der Triage aussortiert (siehe aaa_nicht_aufgenommen.md, aaa_ergebnisse/triage_0X.md).</t>
+          <t>Interne Detailansicht (Tom/Tina v2). Für den Außendienst: aussendienst/AAA_Duesseldorf_2026_Aussendienst.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Ergebnis: 25 GRÜN, 100 GELB, 2 ROT. ALLE Ampeln sind vorläufig: Es gab keinen Browser, kein WebFetch und keine Patentdatenbank, nur Websuche-Treffer. Keine Aussage ist selbst gelesen (Belegstufe V), kein GRÜN ist mailtauglich.</t>
+          <t>Stand 2026-10-15, all about automation Düsseldorf 2026. 127 Firmen geprüft: 25 GRÜN, 100 GELB, 2 ROT. Alle Ampeln vorläufig (kein Browser, keine Patentdatenbank, nur Websuche-Treffer).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>GRÜN bedeutet hier nur: Sitz in DE/AT/NL als erkennbarer Industrie-/Gerätebauer (Sitzregel) plus Produkttyp mit typisch vergossenen/verklebten Bauteilen. Eigenfertigung und Eigenverguss sind nicht belegt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>GELB ist der Normalfall: fehlender Beleg führt nach den v2-Regeln zu Gelb mit Nachrecherche-Auftrag (Spalte J). ROT nur bei hartem Ausschluss (Wettbewerber, Händler, Fertigung außerhalb, CRM-Bestandskunde).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Patentrecherche (Pflicht) bei allen Firmen offen (Google Patents, Espacenet, DEPATISnet nicht erreichbar). Keine Treffer ist kein Befund. Wettbewerbereinsatz meist nur gegen wettbewerber_referenzen.md geprüft.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>CRM-Konzernbezug und Identitätsfragen (Spalte I/J) muss Jey vor jeder Ansprache klären. Nachrecherche mit Browser nachholen.</t>
+          <t>GRÜN = Sitzregel + Produkttyp, Eigenfertigung/Eigenverguss nicht belegt. Patentrecherche offen. CRM-Konzernbezug und Identität vor Kontakt durch Jey klären.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AAA: Demak-Bereich mit klaren Begriffen (Verguss, Verklebung, Dichtung) in beiden Excel-Dateien
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBhay9ftM7ciQ2MUqqBU5G
</commit_message>
<xml_diff>
--- a/aaa_Aussteller_Ampel.xlsx
+++ b/aaa_Aussteller_Ampel.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Optical Bonding (Touch-/HMI-Displays an Handhelds und Safety-Panels), FIPFG/Gasketing (Gehäuse mobiler Geräte), Electrical Insulation …</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Steuer-/Treiberelektronik, Netzteile der Lasersysteme), nachrangig Klebung von Optik/Gehäuse</t>
+          <t>Verguss + Verklebung</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Magnetspulen der Ventile, Ventil-Terminals mit Elektronik, Proportionalventile), nachrangig Gasketing</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Kabelkonfektion, überspritzte/vergossene Steckverbinder, Leiterplatinen, Hybridkabel), nachrangig Gasketing/Sealing …</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich (digitale Montageassistenz, Systemintegration); Randfall Electrical Insulation (IoT-Gateway-Elektronik)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation / E-Mobility Potting (Endprodukt: Zuführ-/Montagemaschinen mit verbauten Antrieben, Sensorik, Steuerungen)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Drucksensoren, Messelektronik, Netzteile in Prüfgeräten), nachrangig Gasketing/Sealing (Dichtheitsprüfung selbst ist …</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Klemmen/Anschlusstechnik für Leistungselektronik, Transformatorenklemmen), nachrangig Gasketing/Sealing (Gehäuse und …</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Heizelemente, Sensorik, Steuerelektronik in Öfen)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Optical Bonding (Panel-PC-Displays, Touch), FIPFG/Gasketing (Gehäuse Rugged Tablets Pokini), nachrangig Electrical Insulation …</t>
+          <t>Verklebung + Dichtung + Verguss</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Encoder/Auswertemodul S.E.M., Antriebselektronik), nachrangig Gasketing/Sealing (IP65-Gehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>LED Encapsulation (LED-Leuchttaster/Leuchtmelder), Electrical Insulation (Not-Halt, RFID, IO-Link-Module), nachrangig Gasketing …</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Optical Bonding (Touch-Keyboards mit Glasfront), FIPFG/Gasketing (IP65-Abdichtung von Industrietastaturen), nachrangig Electrical …</t>
+          <t>Verklebung + Dichtung + Verguss</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (elektrische Greifer, Sensorik, Kontaktmodule), nachrangig Gasketing/Sealing (Durchführungen, Dichtungen)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Sicherheitsrelais, Netzteile, Schaltgeräte, Sensorik), nachrangig Gasketing (IP65-Gehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Elektronikbaugruppen, Steuerungen), nachrangig Gasketing/Sealing (Schaltschrank-/Schutzeinhausungen)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Stromwandler, Messgeräte, Netzteile, Blindleistungsregler), nachrangig E-Mobility/Energie (Messtechnik für Netze)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Mess-/Prüfelektronik, Schaltschränke), nachrangig</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Elektronikbaugruppen, Controller, I/O-Module), nachrangig Gasketing (IP55-Gehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Ventil-/Steuerungselektronik in Handhabungsanlagen), nachrangig Gasketing/Sealing (Pneumatik)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Temperatursensoren/Pyrometer, Messelektronik), nachrangig Gasketing und Optical Bonding (Gehäuse mit Optik/Fenster)</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation / E-Mobility-nah (Gelenkmodule mit Motor, Elektronik, Sensorik); Randbezug: Roboter-Anwendung Dispensing (siehe Feld …</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Steuerplatinen, Netzteile), Optical Bonding (Touch-Bedienterminals)</t>
+          <t>Verguss + Verklebung</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Laserquelle, Steuerelektronik, Netzteil), nachrangig Gasketing (Gehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Joystick-Sensorik, Steuerelektronik), nachrangig Gasketing (IP67-Griffe)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Relais, Netzteile, Schaltgeräte, Elektronik), nachrangig Gasketing/Sealing (Schaltschrank-/Installationsgehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Motor-/Controller-Elektronik der Elektro-Auszüge und Schlösser), nachrangig Gasketing/Klebung</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich. KI-Bildverarbeitung für Qualitätsprüfung (Software), Randfall: Kamera-/Beleuchtungseinheit "AI.SEE Lens" (LED …</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich (Werkstückträger/Handhabung). Randfall: Einbetten/Verkleben von RFID-Chips in Träger</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Antriebs-/Vibrationselektronik, Steuerungen), nachrangig Optical-/Kameramodule</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Bedienterminals/HMI-Elektronik), nachrangig Gasketing/Sealing (Folientastaturen, Gehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation / E-Mobility Potting (Endprodukt: Montage-/Prüfautomaten mit verbauten Antrieben, Sensorik, Steuerungen) …</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Sensorik, Ex-Schutz-Systeme) – nur falls Eigenfertigung</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Schütze, Schaltgeräte, Magnetsysteme/Spulen), nachrangig E-Mobility/PV-DC-Trenner</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Steuerungs-/Panel-Elektronik), nachrangig Gasketing/Sealing (IP-Gehäuse), Optical Bonding (Panels/Displays)</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2654,7 +2654,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Elektronik, Netzteile), nachrangig LED/Sensorik in Kennzeichnungsgeräten</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>unbekannt (Name deutet auf Elektro-Vertrieb)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Magnetventilspulen, Proportionalventile, Ventilinseln mit Elektronik)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Geschäftsbereich (Anlagen-/Maschinenbau; Schaltschrank- und Steuerungsbau nachrangig Electrical Insulation)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Elektronikbaugruppen/Module, Powerline-Modems)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Schaltanlagen, Steuerungen), Gasketing/Sealing (Schaltschrankgehäuse) nur nachrangig</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Embedded-/Industrie-PC-Baugruppen), Optical Bonding (Panel-PCs mit Display, nachrangig), Gasketing (IP-Gehäuse)</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Geschäftsbereich (vermutlich IoT-Plattform/Software)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (überspritzte/vergossene Stecker und Sensor-Aktor-Leitungen), nachrangig Gasketing (IP67-Steckverbinder)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>kein Geschäftsbereich (Handel und Kalibrierdienstleistung)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -3254,7 +3254,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>FIPFG/Gasketing/Sealing (PUR-Gehäusedichtung), nachrangig Optical Bonding (Gehäuse mit Sichtfenster, nicht belegt)</t>
+          <t>Dichtung + Verklebung</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Steckverbinder, vergossene Leitungen, Elektronikbaugruppen), nachrangig FIPFG/Gasketing (Dichtungen)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>FIPFG/Gasketing (Filterlüfter-/Gehäusedichtung), Electrical Insulation (Lüftermotoren, LED-Leuchten, Netzteile), LED Encapsulation …</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Funk-Access-Points/-Clients, Elektronik), nachrangig Gasketing (Gehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Steuer-/I/O-Elektronik), nachrangig Optical Bonding (Panel-PC-Display) und Gasketing (Gehäuse)</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -3554,7 +3554,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (DC-/BLDC-Motoren, Regler), nachrangig E-Mobility Potting (Antriebe, nicht belegt)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Schaltanlagen, verbaute Zukaufteile), nachrangig Gasketing (Schaltschrankgehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Antriebe, Sensorik, Steuerungen in Schleif-/Poliermaschinen), nachrangig Gasketing (Maschinengehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Kabelkonfektion mit vergossenen/überspritzten Steckern, Anschlussleitungen), nachrangig Gasketing …</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Elektronikmodule, Gateways, Embedded-Module), nachrangig Gasketing (Gehäuse IP-Klasse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Motor-/Sensoranbau an Linearachsen), nachrangig Gasketing/Sealing (Dichtungen ATEX-/Reinraumvarianten)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Gasketing/Sealing (Dichteinsätze, Gehäuse), nachrangig Electrical Insulation (Ex-Verschraubungen, Klemmenkästen)</t>
+          <t>Dichtung + Verguss</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>keiner eindeutig (Systemhaus/Sondermaschinenbau); nachrangig Electrical Insulation (Schaltschrank-/Steuerungstechnik)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -4034,7 +4034,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>keiner (Ingenieurdienstleistung); nachrangig Electrical Insulation (Steuerungstechnik für Sondermaschinen)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -4094,7 +4094,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (konfektionierte, überspritzte/vergossene Leitungen, Schrittmotoren, Sensorik), nachrangig Gasketing</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>kein Kerngeschäft (Maschinenbauer); Sekundär: Electrical Insulation (verbaute Steuerungs-/Schaltschrankelektronik), eventuell …</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>keiner (laut Startbase Consulting/B2B-Plattform)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Steuerelektronik, Gateways), Gasketing/Sealing (HMI-Frontdichtung), Optical Bonding (HMI-Panels, Touch-Displays)</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -4334,7 +4334,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (nachrangig; Router-Elektronik mit Schutzlack/Teilverguss)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>kein direkter Bereich; Sekundär: Electrical Insulation (verbaute Steuerungselektronik), Dosier-/Klebezellen als Anlagenbauer (E1 prüfen)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Gasketing/Sealing (luftdichte Dosen, Dichtmanschetten, Dichtungseinsätze), nachrangig Electrical Insulation (Elektronik-Dosen, Brandschutz)</t>
+          <t>Dichtung + Verguss</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>keiner im Kern (Handel); allenfalls Electrical Insulation, falls Kabelkonfektion überspritzt/vergossen</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -4574,7 +4574,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Sensoren, Messsysteme), nur falls in DE gefertigt</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>Kabelverarbeitungs-Maschinenbau; Berührung mit Demak-Kerngeschäft (Dosieren/Vergießen) als Anbieter, nicht als Anwender</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -4694,7 +4694,7 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>Gasketing/Sealing (Schaltschrankbau), Electrical Insulation (Steuerungsbau); Systemintegrator</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
@@ -4754,7 +4754,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Laser-/Steuerelektronik, Netzteile in Lasermarkieranlagen)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Linearmotoren, Servoantriebe), nur falls gefertigt</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Schütze, Relais, Spulen, Netzteile)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>unbekannt</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Wegmesssensorik, Längenmesssysteme)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -5054,7 +5054,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation / Gasketing (IIoT-Router, Gateways in Industriegehäusen)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Kabelkonfektion), nur falls Eigenfertigung</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>nicht bestimmbar</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
@@ -5234,7 +5234,7 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Steckverbinder, konfektionierte Kabel), Gasketing/Sealing (IP67-Steckverbinder)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -5294,7 +5294,7 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Gasketing/Sealing (Schaltschrank-/Elektronikgehäuse), nachrangig Electrical Insulation</t>
+          <t>Dichtung + Verguss</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation / Gasketing (Anlagen- und Schaltschrankelektronik), nachrangig</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>keiner erkennbar (Sondermaschinenbau)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Laser-Netzteile, Steuerelektronik), nachrangig</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Steckverbinder, Kabelbaugruppen, Sensormodule), E-Mobility Potting, Gasketing</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich erkennbar (Produkt unbekannt)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
@@ -5654,7 +5654,7 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Kabelkonfektion mit Hotmelt-Umspritzung, Baugruppen), nachrangig Gasketing</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Servomotoren/Antriebe der Roboter), nachrangig Gasketing (Dichtapplikation durch Roboter ist Anwendung, nicht …</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
@@ -5774,7 +5774,7 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Gasketing/Sealing (Schaltschrankbau), nachrangig Electrical Insulation (Steuerungs- und Antriebstechnik)</t>
+          <t>Dichtung + Verguss</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
@@ -5834,7 +5834,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Kabelkonfektion, Stecker), nachrangig keine</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
@@ -5894,7 +5894,7 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Magnetventilspulen, Ventilelektronik), nachrangig Gasketing/Sealing</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
@@ -5954,7 +5954,7 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Antriebe und Sensorik der Greifer), nachrangig Gasketing</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
@@ -6014,7 +6014,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Optical Bonding / Klebung (Kamera- und Sensorgehäuse), nachrangig Electrical Insulation (Kameraelektronik)</t>
+          <t>Verklebung + Verguss</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
@@ -6074,7 +6074,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich (Sondermaschinenbau); Randfall Electrical Insulation (verbaute Antriebe, Sensorik, Steuerung)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
@@ -6130,7 +6130,7 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich (Visualisierungs-Software mit eigener Hardware "Peakboard Box"); Randfall Electrical Insulation (Embedded-Box)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
@@ -6186,7 +6186,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Signalgeber, Steuerelektronik der Kühlgeräte, Lüfter), LED Encapsulation (LED-Signalleuchten), nachrangig …</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Sicherheitsrelais, Elektronikbaugruppen, Sensoren, Antriebe), nachrangig Gasketing (Gehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr">
@@ -6298,7 +6298,7 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Steuerungs-/Schaltschrankbau, pneumatische/elektrische Antriebe), nachrangig Gasketing/Sealing (Hubtüren)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
@@ -6354,7 +6354,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Optical Bonding (Touch-Systeme/Displays, falls Bonding), Electrical Insulation (Tastatur-/Folienschalter-Elektronik), Gasketing/Sealing …</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (dezentrale Antriebe, Motoren mit Elektronik, Sensorik), nachrangig Gasketing</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr">
@@ -6466,7 +6466,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Sensorkupplungen mit Elektronik), nachrangig Gasketing/Klebung (Kupplungs-Metallmechanik)</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Winden-/Antriebselektronik), nachrangig E-Mobility/Sensorik (Randfall)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>unbekannt (laut Triage evtl. Retrofit/Automation, nicht belegt)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr">
@@ -6634,7 +6634,7 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich; Kabelschutz/Wellrohr-Armaturen, allenfalls Gasketing/Sealing (Verschraubungen, Dichtungen)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Antriebe/Steuerungen der Elektrozylinder und Hubsäulen), nachrangig Gasketing (Gehäuse)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr">
@@ -6754,7 +6754,7 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Sensorik, Steuerelektronik), Randfall</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich (Integrator/Sondermaschinenbau); allenfalls Electrical Insulation (Schaltschränke)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr">
@@ -6874,7 +6874,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Heizelemente, Steuerungen), nachrangig Gasketing (Tür-/Gehäusedichtung)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich (Hydraulikhandel), allenfalls Electrical Insulation (Magnetspulen/Regelelektronik der Partnerfirma)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr">
@@ -6994,7 +6994,7 @@
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Elektromagnetspulen, Steuerelektronik, Akku), nachrangig Gasketing/Klebung</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr">
@@ -7054,7 +7054,7 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>Optical Bonding (Panel-PC/Touch-Displays, nur wenn belegt), Electrical Insulation (Elektronikbaugruppen), Gasketing (IP65-Front)</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr">
@@ -7114,7 +7114,7 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Produktfertigung für Kunden, Sensoren/Elektronik), Gasketing (Gehäuse); Automationsanteil ist Maschinenbau (kein …</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich (Anlagenbau/Montageautomation)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich (Maschinenbau Kabelkonfektion, Schaltschrankbau); allenfalls Electrical Insulation (Schaltschrank-Elektronik)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Handsender-/Empfängerelektronik, Funkmodule), Gasketing/Sealing (Gehäuse IP)</t>
+          <t>Verguss + Dichtung</t>
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr">
@@ -7354,7 +7354,7 @@
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (HF-/Mikrowellenmodule, Thermomanagement) nur bei Eigenfertigung</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Drucktransmitter, Sensorik, Ex-Geräte)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr">
@@ -7474,7 +7474,7 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Steuerelektronik raue Umgebung), Optical Bonding (Industrie-PC mit Display), Gasketing</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr">
@@ -7534,7 +7534,7 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (SPS-Elektronik), nur wenn Fertigung DE/AT/NL; sonst keiner</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr">
@@ -7594,7 +7594,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>unbekannt (vermutlich Bildverarbeitung; kein Bereich ableitbar)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I120" s="2" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Ventil-/Leistungsverstärker, Regelkarten für Hydraulik)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr">
@@ -7714,7 +7714,7 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Encoder, Elektronik, Magnetsensorik), nachrangig Optical Bonding (Displays/Mobile HMI) und Gasketing</t>
+          <t>Verguss + Verklebung + Dichtung</t>
         </is>
       </c>
       <c r="I122" s="2" t="inlineStr">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>keiner erkennbar (Industrievertretung für Komponenten)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I123" s="2" t="inlineStr">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>kein klarer Bereich (Antriebstechnik, PU-Zahnriemen); Gasketing/Doming nur theoretisch</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I124" s="2" t="inlineStr">
@@ -7894,7 +7894,7 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Statorwicklungen, Motorelektronik, Umrichter), E-Mobility Potting nachrangig</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I125" s="2" t="inlineStr">
@@ -7954,7 +7954,7 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Servo- und Umrichter-Leistungselektronik); E-Mobility Potting nachrangig</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>keiner (KI-Software für die Industrie)</t>
+          <t>kein klarer Bereich</t>
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr">
@@ -8066,7 +8066,7 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Electrical Insulation (Drehgeber, Sensorik, Zähler)</t>
+          <t>Verguss</t>
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr">

</xml_diff>